<commit_message>
Update D3S map data
</commit_message>
<xml_diff>
--- a/data/postes_d3s.xlsx
+++ b/data/postes_d3s.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olivierllinares/Documents/01_D3S 2025 2026/DNA 2025 2026/ED3S_Carte_V3_transfert_collegue-2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{654791FF-879C-2E46-BF4B-1236F19A4D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47706A9-9755-6D4C-B1C5-B85F02E56714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="440">
   <si>
     <t>Actif ?</t>
   </si>
@@ -281,9 +281,6 @@
     <t>830015319</t>
   </si>
   <si>
-    <t>Aude</t>
-  </si>
-  <si>
     <t>Occitanie</t>
   </si>
   <si>
@@ -596,21 +593,12 @@
     <t>130042781</t>
   </si>
   <si>
-    <t>directeur adjoint en charge de la qualité, la gestion des risques et référent de la MECS</t>
-  </si>
-  <si>
     <t>Poste réservé aux élèves directeurs - directeur adjoint</t>
   </si>
   <si>
-    <t>établissement Cantoloup Lavallée (Gers)</t>
-  </si>
-  <si>
     <t>Gers</t>
   </si>
   <si>
-    <t>320003544</t>
-  </si>
-  <si>
     <t>https://www.cng.sante.fr/documents/avis-ed3s-2025</t>
   </si>
   <si>
@@ -692,18 +680,6 @@
     <t>940811987</t>
   </si>
   <si>
-    <t>directeur adjoint en charge des finances, de la logistique et de la communication</t>
-  </si>
-  <si>
-    <t>EHPAD « Jean Loubès » à Fanjeaux et EHPAD « Le Garnaguès » à Belpech (direction commune) (Aude)</t>
-  </si>
-  <si>
-    <t>Fanjeaux</t>
-  </si>
-  <si>
-    <t>110780749</t>
-  </si>
-  <si>
     <t>directeur adjoint en charge du suivi de la construction d’un EHPAD site d’Amplepuis, du système d’information en lien avec le GHT</t>
   </si>
   <si>
@@ -1461,6 +1437,45 @@
   </si>
   <si>
     <t>https://www.cng.sante.fr/documents/additif-30/09-ed3s</t>
+  </si>
+  <si>
+    <t>Centre Hospitalier Ariège Couserans</t>
+  </si>
+  <si>
+    <t>Saint Girons</t>
+  </si>
+  <si>
+    <t>Ariege</t>
+  </si>
+  <si>
+    <t>directeur délégué des EHPAD et de l'EPMS</t>
+  </si>
+  <si>
+    <t>090781816</t>
+  </si>
+  <si>
+    <t>EHPAD résidence Docteur Perret</t>
+  </si>
+  <si>
+    <t>Chef d'établissement</t>
+  </si>
+  <si>
+    <t>Directeur</t>
+  </si>
+  <si>
+    <t>5.078651200000077</t>
+  </si>
+  <si>
+    <t>46.457131186241305</t>
+  </si>
+  <si>
+    <t>10000438</t>
+  </si>
+  <si>
+    <t>AURA</t>
+  </si>
+  <si>
+    <t>Saint Trivier de Courtes</t>
   </si>
 </sst>
 </file>
@@ -1468,7 +1483,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="164" formatCode="0.000000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -1525,7 +1540,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1555,7 +1570,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TableauPostes" displayName="TableauPostes" ref="A1:P99">
-  <autoFilter ref="A1:P99" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <autoFilter ref="A1:P99" xr:uid="{00000000-0009-0000-0100-000001000000}">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="Occitanie"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Actif ?"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Poste"/>
@@ -1933,7 +1954,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>16</v>
       </c>
@@ -1941,31 +1962,31 @@
         <v>17</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J2" s="4">
+        <v>45905</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="J2" s="4">
-        <v>45905</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="5">
@@ -1977,7 +1998,7 @@
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
@@ -1985,31 +2006,31 @@
         <v>17</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="J3" s="4">
+        <v>45905</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="J3" s="4">
-        <v>45905</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="5">
@@ -2021,7 +2042,7 @@
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
     </row>
-    <row r="4" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -2029,16 +2050,16 @@
         <v>17</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="F4" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>35</v>
@@ -2047,13 +2068,13 @@
         <v>36</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J4" s="4">
         <v>45905</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="5">
@@ -2065,7 +2086,7 @@
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
     </row>
-    <row r="5" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -2073,31 +2094,31 @@
         <v>17</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>77</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J5" s="4">
         <v>45905</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="5">
@@ -2109,7 +2130,7 @@
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
     </row>
-    <row r="6" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -2117,31 +2138,31 @@
         <v>17</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="4">
+        <v>45905</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="J6" s="4">
-        <v>45905</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="5">
@@ -2153,7 +2174,7 @@
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
     </row>
-    <row r="7" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
@@ -2161,7 +2182,7 @@
         <v>17</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>24</v>
@@ -2185,7 +2206,7 @@
         <v>45905</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="5">
@@ -2197,7 +2218,7 @@
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
     </row>
-    <row r="8" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
@@ -2205,31 +2226,31 @@
         <v>17</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="J8" s="4">
+        <v>45905</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="J8" s="4">
-        <v>45905</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="5">
@@ -2241,7 +2262,7 @@
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
     </row>
-    <row r="9" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -2249,16 +2270,16 @@
         <v>17</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>116</v>
-      </c>
       <c r="F9" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>35</v>
@@ -2267,13 +2288,13 @@
         <v>36</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J9" s="4">
         <v>45905</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L9" s="2"/>
       <c r="M9" s="5">
@@ -2285,7 +2306,7 @@
       <c r="O9" s="2"/>
       <c r="P9" s="2"/>
     </row>
-    <row r="10" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
@@ -2293,16 +2314,16 @@
         <v>17</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>119</v>
-      </c>
       <c r="F10" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>33</v>
@@ -2311,13 +2332,13 @@
         <v>34</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J10" s="4">
         <v>45905</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L10" s="2"/>
       <c r="M10" s="5">
@@ -2329,7 +2350,7 @@
       <c r="O10" s="2"/>
       <c r="P10" s="2"/>
     </row>
-    <row r="11" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>16</v>
       </c>
@@ -2337,31 +2358,31 @@
         <v>17</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>122</v>
-      </c>
       <c r="F11" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J11" s="4">
         <v>45905</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L11" s="2"/>
       <c r="M11" s="5">
@@ -2373,7 +2394,7 @@
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
     </row>
-    <row r="12" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>16</v>
       </c>
@@ -2381,10 +2402,10 @@
         <v>17</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>32</v>
@@ -2397,13 +2418,13 @@
         <v>32</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J12" s="4">
         <v>45905</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L12" s="2"/>
       <c r="M12" s="5">
@@ -2415,7 +2436,7 @@
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
     </row>
-    <row r="13" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
@@ -2423,31 +2444,31 @@
         <v>17</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J13" s="4">
         <v>45905</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L13" s="2"/>
       <c r="M13" s="5">
@@ -2459,7 +2480,7 @@
       <c r="O13" s="2"/>
       <c r="P13" s="2"/>
     </row>
-    <row r="14" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
@@ -2467,31 +2488,31 @@
         <v>17</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="J14" s="4">
+        <v>45905</v>
+      </c>
+      <c r="K14" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="J14" s="4">
-        <v>45905</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="5">
@@ -2503,7 +2524,7 @@
       <c r="O14" s="2"/>
       <c r="P14" s="2"/>
     </row>
-    <row r="15" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>16</v>
       </c>
@@ -2511,31 +2532,31 @@
         <v>17</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="J15" s="4">
+        <v>45905</v>
+      </c>
+      <c r="K15" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="J15" s="4">
-        <v>45905</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="L15" s="2"/>
       <c r="M15" s="5">
@@ -2547,7 +2568,7 @@
       <c r="O15" s="2"/>
       <c r="P15" s="2"/>
     </row>
-    <row r="16" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
@@ -2555,31 +2576,31 @@
         <v>17</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D16" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="F16" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>131</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J16" s="4">
         <v>45905</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="5">
@@ -2591,7 +2612,7 @@
       <c r="O16" s="2"/>
       <c r="P16" s="2"/>
     </row>
-    <row r="17" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -2599,31 +2620,31 @@
         <v>17</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D17" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="F17" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J17" s="4">
         <v>45905</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="5">
@@ -2635,7 +2656,7 @@
       <c r="O17" s="2"/>
       <c r="P17" s="2"/>
     </row>
-    <row r="18" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -2643,16 +2664,16 @@
         <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D18" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="F18" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>33</v>
@@ -2661,13 +2682,13 @@
         <v>34</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J18" s="4">
         <v>45905</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="5">
@@ -2679,7 +2700,7 @@
       <c r="O18" s="2"/>
       <c r="P18" s="2"/>
     </row>
-    <row r="19" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>16</v>
       </c>
@@ -2687,31 +2708,31 @@
         <v>17</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D19" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J19" s="4">
         <v>45905</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="5">
@@ -2723,7 +2744,7 @@
       <c r="O19" s="2"/>
       <c r="P19" s="2"/>
     </row>
-    <row r="20" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
@@ -2731,31 +2752,31 @@
         <v>17</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="J20" s="4">
+        <v>45905</v>
+      </c>
+      <c r="K20" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="J20" s="4">
-        <v>45905</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="5">
@@ -2767,7 +2788,7 @@
       <c r="O20" s="2"/>
       <c r="P20" s="2"/>
     </row>
-    <row r="21" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>16</v>
       </c>
@@ -2775,10 +2796,10 @@
         <v>17</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>20</v>
@@ -2799,7 +2820,7 @@
         <v>45905</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="5">
@@ -2811,7 +2832,7 @@
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
     </row>
-    <row r="22" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>16</v>
       </c>
@@ -2819,7 +2840,7 @@
         <v>17</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>37</v>
@@ -2841,7 +2862,7 @@
         <v>45905</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="5">
@@ -2853,7 +2874,7 @@
       <c r="O22" s="2"/>
       <c r="P22" s="2"/>
     </row>
-    <row r="23" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>16</v>
       </c>
@@ -2861,31 +2882,31 @@
         <v>17</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D23" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="F23" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J23" s="4">
         <v>45905</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="5">
@@ -2897,7 +2918,7 @@
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
     </row>
-    <row r="24" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>16</v>
       </c>
@@ -2905,16 +2926,16 @@
         <v>17</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D24" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>142</v>
-      </c>
       <c r="F24" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>33</v>
@@ -2923,13 +2944,13 @@
         <v>34</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J24" s="4">
         <v>45905</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="5">
@@ -2941,7 +2962,7 @@
       <c r="O24" s="2"/>
       <c r="P24" s="2"/>
     </row>
-    <row r="25" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>16</v>
       </c>
@@ -2949,29 +2970,29 @@
         <v>17</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H25" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J25" s="4">
         <v>45905</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="5">
@@ -2983,7 +3004,7 @@
       <c r="O25" s="2"/>
       <c r="P25" s="2"/>
     </row>
-    <row r="26" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>16</v>
       </c>
@@ -2991,31 +3012,31 @@
         <v>17</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="F26" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J26" s="4">
         <v>45905</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="5">
@@ -3027,81 +3048,83 @@
       <c r="O26" s="2"/>
       <c r="P26" s="2"/>
     </row>
-    <row r="27" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>146</v>
+        <v>430</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>148</v>
+        <v>427</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="F27" s="2"/>
+        <v>428</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>428</v>
+      </c>
       <c r="G27" s="2" t="s">
-        <v>149</v>
+        <v>429</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>150</v>
+        <v>431</v>
       </c>
       <c r="J27" s="4">
-        <v>45905</v>
+        <v>46204</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L27" s="2"/>
       <c r="M27" s="5">
-        <v>43.69</v>
+        <v>42.999463900000002</v>
       </c>
       <c r="N27" s="5">
-        <v>0.45</v>
+        <v>1.1317678</v>
       </c>
       <c r="O27" s="2"/>
       <c r="P27" s="2"/>
     </row>
-    <row r="28" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="I28" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>156</v>
-      </c>
       <c r="J28" s="4">
         <v>45905</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L28" s="2"/>
       <c r="M28" s="5">
@@ -3113,24 +3136,24 @@
       <c r="O28" s="2"/>
       <c r="P28" s="2"/>
     </row>
-    <row r="29" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>29</v>
@@ -3139,13 +3162,13 @@
         <v>30</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="J29" s="4">
         <v>45905</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L29" s="2"/>
       <c r="M29" s="5">
@@ -3157,39 +3180,39 @@
       <c r="O29" s="2"/>
       <c r="P29" s="2"/>
     </row>
-    <row r="30" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="J30" s="4">
         <v>45905</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L30" s="2"/>
       <c r="M30" s="5">
@@ -3201,39 +3224,39 @@
       <c r="O30" s="2"/>
       <c r="P30" s="2"/>
     </row>
-    <row r="31" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="J31" s="4">
         <v>45905</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L31" s="2"/>
       <c r="M31" s="5">
@@ -3245,39 +3268,39 @@
       <c r="O31" s="2"/>
       <c r="P31" s="2"/>
     </row>
-    <row r="32" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="J32" s="4">
         <v>45905</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L32" s="2"/>
       <c r="M32" s="5">
@@ -3289,37 +3312,37 @@
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
     </row>
-    <row r="33" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="J33" s="4">
         <v>45905</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L33" s="2"/>
       <c r="M33" s="5">
@@ -3331,83 +3354,83 @@
       <c r="O33" s="2"/>
       <c r="P33" s="2"/>
     </row>
-    <row r="34" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>178</v>
+        <v>434</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>147</v>
+        <v>433</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>179</v>
+        <v>432</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>180</v>
+        <v>439</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>180</v>
+        <v>439</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>42</v>
+        <v>438</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>181</v>
+        <v>437</v>
       </c>
       <c r="J34" s="4">
-        <v>45905</v>
+        <v>46204</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L34" s="2"/>
-      <c r="M34" s="5">
-        <v>43.1</v>
-      </c>
-      <c r="N34" s="5">
-        <v>2.41</v>
+      <c r="M34" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="N34" s="5" t="s">
+        <v>435</v>
       </c>
       <c r="O34" s="2"/>
       <c r="P34" s="2"/>
     </row>
-    <row r="35" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="J35" s="4">
         <v>45905</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L35" s="2"/>
       <c r="M35" s="5">
@@ -3419,24 +3442,24 @@
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
     </row>
-    <row r="36" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>31</v>
@@ -3445,13 +3468,13 @@
         <v>30</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="J36" s="4">
         <v>45905</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L36" s="2"/>
       <c r="M36" s="5">
@@ -3463,18 +3486,18 @@
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
     </row>
-    <row r="37" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>33</v>
@@ -3487,13 +3510,13 @@
         <v>34</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="J37" s="4">
         <v>45905</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L37" s="2"/>
       <c r="M37" s="5">
@@ -3505,39 +3528,39 @@
       <c r="O37" s="2"/>
       <c r="P37" s="2"/>
     </row>
-    <row r="38" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="J38" s="4">
         <v>45905</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L38" s="2"/>
       <c r="M38" s="5">
@@ -3549,39 +3572,39 @@
       <c r="O38" s="2"/>
       <c r="P38" s="2"/>
     </row>
-    <row r="39" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="J39" s="4">
         <v>45905</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L39" s="2"/>
       <c r="M39" s="5">
@@ -3593,39 +3616,39 @@
       <c r="O39" s="2"/>
       <c r="P39" s="2"/>
     </row>
-    <row r="40" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="J40" s="4">
         <v>45905</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L40" s="2"/>
       <c r="M40" s="5">
@@ -3637,37 +3660,37 @@
       <c r="O40" s="2"/>
       <c r="P40" s="2"/>
     </row>
-    <row r="41" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="J41" s="4">
         <v>45905</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L41" s="2"/>
       <c r="M41" s="5">
@@ -3679,39 +3702,39 @@
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>
     </row>
-    <row r="42" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:16" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="J42" s="4">
         <v>45905</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L42" s="2"/>
       <c r="M42" s="5">
@@ -3723,39 +3746,39 @@
       <c r="O42" s="2"/>
       <c r="P42" s="2"/>
     </row>
-    <row r="43" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="J43" s="4">
         <v>45905</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L43" s="2"/>
       <c r="M43" s="5">
@@ -3767,39 +3790,39 @@
       <c r="O43" s="2"/>
       <c r="P43" s="2"/>
     </row>
-    <row r="44" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="J44" s="4">
         <v>45905</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L44" s="2"/>
       <c r="M44" s="5">
@@ -3811,39 +3834,39 @@
       <c r="O44" s="2"/>
       <c r="P44" s="2"/>
     </row>
-    <row r="45" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I45" s="3" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="J45" s="4">
         <v>45905</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L45" s="2"/>
       <c r="M45" s="5">
@@ -3855,39 +3878,39 @@
       <c r="O45" s="2"/>
       <c r="P45" s="2"/>
     </row>
-    <row r="46" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="G46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H46" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H46" s="2" t="s">
-        <v>50</v>
-      </c>
       <c r="I46" s="3" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="J46" s="4">
         <v>45905</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L46" s="2"/>
       <c r="M46" s="5">
@@ -3899,39 +3922,39 @@
       <c r="O46" s="2"/>
       <c r="P46" s="2"/>
     </row>
-    <row r="47" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:16" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="J47" s="4">
         <v>45905</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L47" s="2"/>
       <c r="M47" s="5">
@@ -3943,24 +3966,24 @@
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
     </row>
-    <row r="48" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:16" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>29</v>
@@ -3969,13 +3992,13 @@
         <v>30</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="J48" s="4">
         <v>45905</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L48" s="2"/>
       <c r="M48" s="5">
@@ -3987,18 +4010,18 @@
       <c r="O48" s="2"/>
       <c r="P48" s="2"/>
     </row>
-    <row r="49" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>21</v>
@@ -4011,13 +4034,13 @@
         <v>22</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="J49" s="4">
         <v>45905</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L49" s="2"/>
       <c r="M49" s="5">
@@ -4034,34 +4057,34 @@
         <v>16</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="J50" s="4">
         <v>45905</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L50" s="2"/>
       <c r="M50" s="5">
@@ -4073,24 +4096,24 @@
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
     </row>
-    <row r="51" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>29</v>
@@ -4099,13 +4122,13 @@
         <v>30</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="J51" s="4">
         <v>45905</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L51" s="2"/>
       <c r="M51" s="5">
@@ -4117,37 +4140,37 @@
       <c r="O51" s="2"/>
       <c r="P51" s="2"/>
     </row>
-    <row r="52" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F52" s="2"/>
       <c r="G52" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H52" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H52" s="2" t="s">
+      <c r="I52" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I52" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="J52" s="4">
         <v>45905</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L52" s="2"/>
       <c r="M52" s="5">
@@ -4159,24 +4182,24 @@
       <c r="O52" s="2"/>
       <c r="P52" s="2"/>
     </row>
-    <row r="53" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:16" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>21</v>
@@ -4185,13 +4208,13 @@
         <v>22</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="J53" s="4">
         <v>45905</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L53" s="2"/>
       <c r="M53" s="5">
@@ -4203,39 +4226,39 @@
       <c r="O53" s="2"/>
       <c r="P53" s="2"/>
     </row>
-    <row r="54" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H54" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J54" s="4">
         <v>45905</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L54" s="2"/>
       <c r="M54" s="5">
@@ -4247,39 +4270,39 @@
       <c r="O54" s="2"/>
       <c r="P54" s="2"/>
     </row>
-    <row r="55" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="J55" s="4">
         <v>45905</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L55" s="2"/>
       <c r="M55" s="5">
@@ -4291,39 +4314,39 @@
       <c r="O55" s="2"/>
       <c r="P55" s="2"/>
     </row>
-    <row r="56" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:16" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="J56" s="4">
         <v>45905</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L56" s="2"/>
       <c r="M56" s="5">
@@ -4335,18 +4358,18 @@
       <c r="O56" s="2"/>
       <c r="P56" s="2"/>
     </row>
-    <row r="57" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>21</v>
@@ -4359,13 +4382,13 @@
         <v>22</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="J57" s="4">
         <v>45905</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L57" s="2"/>
       <c r="M57" s="5">
@@ -4377,39 +4400,39 @@
       <c r="O57" s="2"/>
       <c r="P57" s="2"/>
     </row>
-    <row r="58" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:16" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="J58" s="4">
         <v>45905</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L58" s="2"/>
       <c r="M58" s="5">
@@ -4421,37 +4444,37 @@
       <c r="O58" s="2"/>
       <c r="P58" s="2"/>
     </row>
-    <row r="59" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="F59" s="2"/>
       <c r="G59" s="2" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="J59" s="4">
         <v>45905</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L59" s="2"/>
       <c r="M59" s="5">
@@ -4463,39 +4486,39 @@
       <c r="O59" s="2"/>
       <c r="P59" s="2"/>
     </row>
-    <row r="60" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="J60" s="4">
         <v>45905</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L60" s="2"/>
       <c r="M60" s="5">
@@ -4507,24 +4530,24 @@
       <c r="O60" s="2"/>
       <c r="P60" s="2"/>
     </row>
-    <row r="61" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>33</v>
@@ -4533,13 +4556,13 @@
         <v>34</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="J61" s="4">
         <v>45905</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L61" s="2"/>
       <c r="M61" s="5">
@@ -4551,24 +4574,24 @@
       <c r="O61" s="2"/>
       <c r="P61" s="2"/>
     </row>
-    <row r="62" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>18</v>
@@ -4577,13 +4600,13 @@
         <v>19</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="J62" s="4">
         <v>45905</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L62" s="2"/>
       <c r="M62" s="5">
@@ -4595,39 +4618,39 @@
       <c r="O62" s="2"/>
       <c r="P62" s="2"/>
     </row>
-    <row r="63" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="J63" s="4">
         <v>45905</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L63" s="2"/>
       <c r="M63" s="5">
@@ -4639,39 +4662,39 @@
       <c r="O63" s="2"/>
       <c r="P63" s="2"/>
     </row>
-    <row r="64" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="J64" s="4">
         <v>45905</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L64" s="2"/>
       <c r="M64" s="5">
@@ -4683,37 +4706,37 @@
       <c r="O64" s="2"/>
       <c r="P64" s="2"/>
     </row>
-    <row r="65" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="F65" s="2"/>
       <c r="G65" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="H65" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J65" s="4">
         <v>45905</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L65" s="2"/>
       <c r="M65" s="5">
@@ -4725,39 +4748,39 @@
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
     </row>
-    <row r="66" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:16" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="J66" s="4">
         <v>45905</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L66" s="2"/>
       <c r="M66" s="5">
@@ -4769,24 +4792,24 @@
       <c r="O66" s="2"/>
       <c r="P66" s="2"/>
     </row>
-    <row r="67" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="G67" s="2" t="s">
         <v>21</v>
@@ -4795,13 +4818,13 @@
         <v>22</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="J67" s="4">
         <v>45905</v>
       </c>
       <c r="K67" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L67" s="2"/>
       <c r="M67" s="5">
@@ -4813,39 +4836,39 @@
       <c r="O67" s="2"/>
       <c r="P67" s="2"/>
     </row>
-    <row r="68" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="I68" s="3" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="J68" s="4">
         <v>45905</v>
       </c>
       <c r="K68" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L68" s="2"/>
       <c r="M68" s="5">
@@ -4857,39 +4880,39 @@
       <c r="O68" s="2"/>
       <c r="P68" s="2"/>
     </row>
-    <row r="69" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:16" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="H69" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="J69" s="4">
         <v>45905</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L69" s="2"/>
       <c r="M69" s="5">
@@ -4906,34 +4929,34 @@
         <v>16</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="J70" s="4">
         <v>45905</v>
       </c>
       <c r="K70" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L70" s="2"/>
       <c r="M70" s="5">
@@ -4945,39 +4968,39 @@
       <c r="O70" s="2"/>
       <c r="P70" s="2"/>
     </row>
-    <row r="71" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:16" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>34</v>
       </c>
       <c r="I71" s="3" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="J71" s="4">
         <v>45905</v>
       </c>
       <c r="K71" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L71" s="2"/>
       <c r="M71" s="5">
@@ -4989,39 +5012,39 @@
       <c r="O71" s="2"/>
       <c r="P71" s="2"/>
     </row>
-    <row r="72" spans="1:16" ht="112" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:16" ht="112" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I72" s="3" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="J72" s="4">
         <v>45905</v>
       </c>
       <c r="K72" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L72" s="2"/>
       <c r="M72" s="5">
@@ -5033,24 +5056,24 @@
       <c r="O72" s="2"/>
       <c r="P72" s="2"/>
     </row>
-    <row r="73" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="G73" s="2" t="s">
         <v>38</v>
@@ -5059,13 +5082,13 @@
         <v>39</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="J73" s="4">
         <v>45905</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L73" s="2"/>
       <c r="M73" s="5">
@@ -5077,39 +5100,39 @@
       <c r="O73" s="2"/>
       <c r="P73" s="2"/>
     </row>
-    <row r="74" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:16" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="J74" s="4">
         <v>45905</v>
       </c>
       <c r="K74" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L74" s="2"/>
       <c r="M74" s="5">
@@ -5121,39 +5144,39 @@
       <c r="O74" s="2"/>
       <c r="P74" s="2"/>
     </row>
-    <row r="75" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="H75" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="J75" s="4">
         <v>45905</v>
       </c>
       <c r="K75" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L75" s="2"/>
       <c r="M75" s="5">
@@ -5165,39 +5188,39 @@
       <c r="O75" s="2"/>
       <c r="P75" s="2"/>
     </row>
-    <row r="76" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="H76" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="J76" s="4">
         <v>45905</v>
       </c>
       <c r="K76" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L76" s="2"/>
       <c r="M76" s="5">
@@ -5209,39 +5232,39 @@
       <c r="O76" s="2"/>
       <c r="P76" s="2"/>
     </row>
-    <row r="77" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="G77" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="H77" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="H77" s="2" t="s">
-        <v>89</v>
-      </c>
       <c r="I77" s="3" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="J77" s="4">
         <v>45905</v>
       </c>
       <c r="K77" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L77" s="2"/>
       <c r="M77" s="5">
@@ -5253,39 +5276,39 @@
       <c r="O77" s="2"/>
       <c r="P77" s="2"/>
     </row>
-    <row r="78" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:16" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H78" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="J78" s="4">
         <v>45905</v>
       </c>
       <c r="K78" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L78" s="2"/>
       <c r="M78" s="5">
@@ -5297,39 +5320,39 @@
       <c r="O78" s="2"/>
       <c r="P78" s="2"/>
     </row>
-    <row r="79" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:16" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H79" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="J79" s="4">
         <v>45905</v>
       </c>
       <c r="K79" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L79" s="2"/>
       <c r="M79" s="5">
@@ -5346,34 +5369,34 @@
         <v>16</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I80" s="3" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="J80" s="4">
         <v>45905</v>
       </c>
       <c r="K80" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L80" s="2"/>
       <c r="M80" s="5">
@@ -5385,39 +5408,39 @@
       <c r="O80" s="2"/>
       <c r="P80" s="2"/>
     </row>
-    <row r="81" spans="1:16" ht="96" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:16" ht="96" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I81" s="3" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="J81" s="4">
         <v>45905</v>
       </c>
       <c r="K81" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L81" s="2"/>
       <c r="M81" s="5">
@@ -5429,39 +5452,39 @@
       <c r="O81" s="2"/>
       <c r="P81" s="2"/>
     </row>
-    <row r="82" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I82" s="3" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="J82" s="4">
         <v>45905</v>
       </c>
       <c r="K82" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L82" s="2"/>
       <c r="M82" s="5">
@@ -5473,39 +5496,39 @@
       <c r="O82" s="2"/>
       <c r="P82" s="2"/>
     </row>
-    <row r="83" spans="1:16" ht="112" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:16" ht="112" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="J83" s="4">
         <v>45905</v>
       </c>
       <c r="K83" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L83" s="2"/>
       <c r="M83" s="5">
@@ -5517,37 +5540,37 @@
       <c r="O83" s="2"/>
       <c r="P83" s="2"/>
     </row>
-    <row r="84" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="F84" s="2"/>
       <c r="G84" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="H84" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="J84" s="4">
         <v>45905</v>
       </c>
       <c r="K84" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L84" s="2"/>
       <c r="M84" s="5">
@@ -5559,39 +5582,39 @@
       <c r="O84" s="2"/>
       <c r="P84" s="2"/>
     </row>
-    <row r="85" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H85" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I85" s="3" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="J85" s="4">
         <v>45905</v>
       </c>
       <c r="K85" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L85" s="2"/>
       <c r="M85" s="5">
@@ -5603,39 +5626,39 @@
       <c r="O85" s="2"/>
       <c r="P85" s="2"/>
     </row>
-    <row r="86" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:16" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H86" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J86" s="4">
         <v>45905</v>
       </c>
       <c r="K86" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L86" s="2"/>
       <c r="M86" s="5">
@@ -5647,39 +5670,39 @@
       <c r="O86" s="2"/>
       <c r="P86" s="2"/>
     </row>
-    <row r="87" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:16" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>378</v>
+        <v>370</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>379</v>
+        <v>371</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="H87" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="J87" s="4">
         <v>45905</v>
       </c>
       <c r="K87" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L87" s="2"/>
       <c r="M87" s="5">
@@ -5696,34 +5719,34 @@
         <v>16</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>380</v>
+        <v>372</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>381</v>
+        <v>373</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>382</v>
+        <v>374</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>382</v>
+        <v>374</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>383</v>
+        <v>375</v>
       </c>
       <c r="H88" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="J88" s="4">
         <v>45905</v>
       </c>
       <c r="K88" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L88" s="2"/>
       <c r="M88" s="5">
@@ -5735,39 +5758,39 @@
       <c r="O88" s="2"/>
       <c r="P88" s="2"/>
     </row>
-    <row r="89" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:16" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>386</v>
+        <v>378</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H89" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="J89" s="4">
         <v>45905</v>
       </c>
       <c r="K89" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L89" s="2"/>
       <c r="M89" s="5">
@@ -5779,39 +5802,39 @@
       <c r="O89" s="2"/>
       <c r="P89" s="2"/>
     </row>
-    <row r="90" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
       <c r="H90" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="J90" s="4">
         <v>45905</v>
       </c>
       <c r="K90" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L90" s="2"/>
       <c r="M90" s="5">
@@ -5823,39 +5846,39 @@
       <c r="O90" s="2"/>
       <c r="P90" s="2"/>
     </row>
-    <row r="91" spans="1:16" ht="80" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:16" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H91" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
       <c r="J91" s="4">
         <v>45905</v>
       </c>
       <c r="K91" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L91" s="2"/>
       <c r="M91" s="5">
@@ -5867,18 +5890,18 @@
       <c r="O91" s="2"/>
       <c r="P91" s="2"/>
     </row>
-    <row r="92" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:16" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>399</v>
+        <v>391</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>21</v>
@@ -5891,13 +5914,13 @@
         <v>22</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="J92" s="4">
         <v>45905</v>
       </c>
       <c r="K92" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L92" s="2"/>
       <c r="M92" s="5">
@@ -5909,39 +5932,39 @@
       <c r="O92" s="2"/>
       <c r="P92" s="2"/>
     </row>
-    <row r="93" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>401</v>
+        <v>393</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>402</v>
+        <v>394</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I93" s="3" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="J93" s="4">
         <v>45905</v>
       </c>
       <c r="K93" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L93" s="2"/>
       <c r="M93" s="5">
@@ -5953,39 +5976,39 @@
       <c r="O93" s="2"/>
       <c r="P93" s="2"/>
     </row>
-    <row r="94" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:16" ht="64" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
       <c r="H94" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I94" s="3" t="s">
-        <v>408</v>
+        <v>400</v>
       </c>
       <c r="J94" s="4">
         <v>45905</v>
       </c>
       <c r="K94" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="L94" s="2"/>
       <c r="M94" s="5">
@@ -5997,39 +6020,39 @@
       <c r="O94" s="2"/>
       <c r="P94" s="2"/>
     </row>
-    <row r="95" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>409</v>
+        <v>401</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>410</v>
+        <v>402</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>411</v>
+        <v>403</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>411</v>
+        <v>403</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>412</v>
+        <v>404</v>
       </c>
       <c r="I95" s="3" t="s">
-        <v>413</v>
+        <v>405</v>
       </c>
       <c r="J95" s="4">
         <v>45909</v>
       </c>
       <c r="K95" s="2" t="s">
-        <v>414</v>
+        <v>406</v>
       </c>
       <c r="L95" s="2"/>
       <c r="M95" s="5">
@@ -6041,39 +6064,39 @@
       <c r="O95" s="2"/>
       <c r="P95" s="2"/>
     </row>
-    <row r="96" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="E96" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G96" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="F96" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="G96" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="H96" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I96" s="3" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="J96" s="4">
         <v>45912</v>
       </c>
       <c r="K96" s="2" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="L96" s="2"/>
       <c r="M96" s="5">
@@ -6085,42 +6108,42 @@
       <c r="O96" s="2"/>
       <c r="P96" s="2"/>
     </row>
-    <row r="97" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="H97" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I97" s="3" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="J97" s="4">
         <v>45917</v>
       </c>
       <c r="K97" s="2" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="L97" s="2" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
       <c r="M97" s="5">
         <v>49.1</v>
@@ -6131,39 +6154,39 @@
       <c r="O97" s="2"/>
       <c r="P97" s="2"/>
     </row>
-    <row r="98" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:16" ht="48" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="H98" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I98" s="3" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
       <c r="J98" s="4">
         <v>45920</v>
       </c>
       <c r="K98" s="2" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
       <c r="L98" s="2"/>
       <c r="M98" s="5">
@@ -6180,34 +6203,34 @@
         <v>16</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>430</v>
+        <v>422</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="H99" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I99" s="3" t="s">
-        <v>433</v>
+        <v>425</v>
       </c>
       <c r="J99" s="4">
         <v>45928</v>
       </c>
       <c r="K99" s="2" t="s">
-        <v>434</v>
+        <v>426</v>
       </c>
       <c r="L99" s="2"/>
       <c r="M99" s="5">

</xml_diff>

<commit_message>
Correct Draguignan post locations
</commit_message>
<xml_diff>
--- a/data/postes_d3s.xlsx
+++ b/data/postes_d3s.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olivierllinares/Documents/01_D3S 2025 2026/DNA 2025 2026/ED3S_Carte_V3_transfert_collegue-2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0A23492-D62C-5441-83B8-E15A2282B132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB84316F-0751-5A48-8113-17B2FA4240D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -147,7 +147,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1176" uniqueCount="664">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1174" uniqueCount="663">
   <si>
     <t>Actif ?</t>
   </si>
@@ -1848,21 +1848,12 @@
     <t>2.253651598062639</t>
   </si>
   <si>
-    <t>830000600</t>
-  </si>
-  <si>
     <t>Centre départemental de l'enfance (draguignan)</t>
   </si>
   <si>
     <t>Draguignan</t>
   </si>
   <si>
-    <t xml:space="preserve">43.54444616987069   </t>
-  </si>
-  <si>
-    <t>6.463231746883476</t>
-  </si>
-  <si>
     <t>860792993</t>
   </si>
   <si>
@@ -2140,6 +2131,12 @@
   </si>
   <si>
     <t>Directeur du pôle éducatif poste 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43.54524606024483  </t>
+  </si>
+  <si>
+    <t>6.463718909248732</t>
   </si>
 </sst>
 </file>
@@ -3187,10 +3184,10 @@
         <v>142</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>50</v>
@@ -3209,10 +3206,10 @@
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="5" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="O14" s="2"/>
       <c r="P14" s="2"/>
@@ -6140,19 +6137,19 @@
         <v>16</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D81" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="E81" s="2" t="s">
         <v>567</v>
       </c>
-      <c r="E81" s="2" t="s">
-        <v>568</v>
-      </c>
       <c r="F81" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="G81" s="2" t="s">
         <v>29</v>
@@ -6160,9 +6157,7 @@
       <c r="H81" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="I81" s="3" t="s">
-        <v>566</v>
-      </c>
+      <c r="I81" s="3"/>
       <c r="J81" s="4">
         <v>46258</v>
       </c>
@@ -6171,10 +6166,10 @@
       </c>
       <c r="L81" s="2"/>
       <c r="M81" s="5" t="s">
-        <v>569</v>
+        <v>661</v>
       </c>
       <c r="N81" s="5" t="s">
-        <v>570</v>
+        <v>662</v>
       </c>
       <c r="O81" s="2"/>
       <c r="P81" s="2"/>
@@ -6184,19 +6179,19 @@
         <v>16</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D82" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="E82" s="2" t="s">
         <v>567</v>
       </c>
-      <c r="E82" s="2" t="s">
-        <v>568</v>
-      </c>
       <c r="F82" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="G82" s="2" t="s">
         <v>29</v>
@@ -6204,9 +6199,7 @@
       <c r="H82" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="I82" s="3" t="s">
-        <v>566</v>
-      </c>
+      <c r="I82" s="3"/>
       <c r="J82" s="4">
         <v>46258</v>
       </c>
@@ -6215,10 +6208,10 @@
       </c>
       <c r="L82" s="2"/>
       <c r="M82" s="5" t="s">
-        <v>569</v>
+        <v>661</v>
       </c>
       <c r="N82" s="5" t="s">
-        <v>570</v>
+        <v>662</v>
       </c>
       <c r="O82" s="2"/>
       <c r="P82" s="2"/>
@@ -6228,28 +6221,28 @@
         <v>16</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="H83" s="2" t="s">
         <v>24</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="J83" s="4">
         <v>46258</v>
@@ -6259,10 +6252,10 @@
       </c>
       <c r="L83" s="2"/>
       <c r="M83" s="5" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="N83" s="5" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="O83" s="2"/>
       <c r="P83" s="2"/>
@@ -6272,19 +6265,19 @@
         <v>16</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="G84" s="2" t="s">
         <v>38</v>
@@ -6293,7 +6286,7 @@
         <v>24</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="J84" s="4">
         <v>46258</v>
@@ -6303,10 +6296,10 @@
       </c>
       <c r="L84" s="2"/>
       <c r="M84" s="5" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="N84" s="5" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="O84" s="2"/>
       <c r="P84" s="2"/>
@@ -6322,13 +6315,13 @@
         <v>70</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>38</v>
@@ -6337,7 +6330,7 @@
         <v>24</v>
       </c>
       <c r="I85" s="3" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="J85" s="4">
         <v>46258</v>
@@ -6347,10 +6340,10 @@
       </c>
       <c r="L85" s="2"/>
       <c r="M85" s="5" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="N85" s="5" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="O85" s="2"/>
       <c r="P85" s="2"/>
@@ -6366,13 +6359,13 @@
         <v>70</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="G86" s="2" t="s">
         <v>38</v>
@@ -6381,7 +6374,7 @@
         <v>24</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="J86" s="4">
         <v>46258</v>
@@ -6391,10 +6384,10 @@
       </c>
       <c r="L86" s="2"/>
       <c r="M86" s="5" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="N86" s="5" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="O86" s="2"/>
       <c r="P86" s="2"/>
@@ -6404,19 +6397,19 @@
         <v>16</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="C87" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D87" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="E87" s="2" t="s">
         <v>591</v>
       </c>
-      <c r="E87" s="2" t="s">
-        <v>594</v>
-      </c>
       <c r="F87" s="2" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>37</v>
@@ -6425,7 +6418,7 @@
         <v>32</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="J87" s="4">
         <v>46258</v>
@@ -6434,13 +6427,13 @@
         <v>49</v>
       </c>
       <c r="L87" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="M87" s="5" t="s">
         <v>593</v>
       </c>
-      <c r="M87" s="5" t="s">
-        <v>596</v>
-      </c>
       <c r="N87" s="5" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="O87" s="2"/>
       <c r="P87" s="2"/>
@@ -6450,19 +6443,19 @@
         <v>16</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>37</v>
@@ -6471,7 +6464,7 @@
         <v>32</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="J88" s="4">
         <v>46258</v>
@@ -6481,10 +6474,10 @@
       </c>
       <c r="L88" s="2"/>
       <c r="M88" s="5" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="N88" s="5" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="O88" s="2"/>
       <c r="P88" s="2"/>
@@ -6494,28 +6487,28 @@
         <v>16</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="H89" s="2" t="s">
         <v>32</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="J89" s="4">
         <v>46258</v>
@@ -6525,10 +6518,10 @@
       </c>
       <c r="L89" s="2"/>
       <c r="M89" s="5" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="N89" s="5" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="O89" s="2"/>
       <c r="P89" s="2"/>
@@ -6538,19 +6531,19 @@
         <v>16</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="C90" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>57</v>
@@ -6559,7 +6552,7 @@
         <v>520</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="J90" s="4">
         <v>46258</v>
@@ -6568,13 +6561,13 @@
         <v>49</v>
       </c>
       <c r="L90" s="2" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="M90" s="5" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="N90" s="5" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="O90" s="2"/>
       <c r="P90" s="2"/>
@@ -6584,19 +6577,19 @@
         <v>16</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="C91" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>57</v>
@@ -6605,7 +6598,7 @@
         <v>520</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="J91" s="4">
         <v>46258</v>
@@ -6615,10 +6608,10 @@
       </c>
       <c r="L91" s="2"/>
       <c r="M91" s="5" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="N91" s="5" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="O91" s="2"/>
       <c r="P91" s="2"/>
@@ -6628,19 +6621,19 @@
         <v>16</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="C92" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D92" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="E92" s="2" t="s">
         <v>626</v>
       </c>
-      <c r="E92" s="2" t="s">
-        <v>629</v>
-      </c>
       <c r="F92" s="2" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="G92" s="2" t="s">
         <v>57</v>
@@ -6649,7 +6642,7 @@
         <v>520</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="J92" s="4">
         <v>46258</v>
@@ -6658,13 +6651,13 @@
         <v>49</v>
       </c>
       <c r="L92" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="M92" s="5" t="s">
+        <v>627</v>
+      </c>
+      <c r="N92" s="5" t="s">
         <v>628</v>
-      </c>
-      <c r="M92" s="5" t="s">
-        <v>630</v>
-      </c>
-      <c r="N92" s="5" t="s">
-        <v>631</v>
       </c>
       <c r="O92" s="2"/>
       <c r="P92" s="2"/>
@@ -6674,19 +6667,19 @@
         <v>16</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="C93" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>57</v>
@@ -6695,7 +6688,7 @@
         <v>520</v>
       </c>
       <c r="I93" s="3" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="J93" s="4">
         <v>46258</v>
@@ -6705,10 +6698,10 @@
       </c>
       <c r="L93" s="2"/>
       <c r="M93" s="5" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="N93" s="5" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="O93" s="2"/>
       <c r="P93" s="2"/>
@@ -6718,28 +6711,28 @@
         <v>16</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D94" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="G94" s="2" t="s">
         <v>639</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>641</v>
-      </c>
-      <c r="F94" s="2" t="s">
-        <v>641</v>
-      </c>
-      <c r="G94" s="2" t="s">
-        <v>642</v>
       </c>
       <c r="H94" s="2" t="s">
         <v>520</v>
       </c>
       <c r="I94" s="3" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="J94" s="4">
         <v>46258</v>
@@ -6748,13 +6741,13 @@
         <v>49</v>
       </c>
       <c r="L94" s="2" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="M94" s="5" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="N94" s="5" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="O94" s="2"/>
       <c r="P94" s="2"/>
@@ -6764,28 +6757,28 @@
         <v>16</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="C95" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="H95" s="2" t="s">
         <v>520</v>
       </c>
       <c r="I95" s="3" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="J95" s="4">
         <v>46258</v>
@@ -6794,13 +6787,13 @@
         <v>60</v>
       </c>
       <c r="L95" s="2" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="M95" s="5" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="N95" s="5" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="O95" s="2"/>
       <c r="P95" s="2"/>
@@ -6810,19 +6803,19 @@
         <v>16</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>77</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="G96" s="2" t="s">
         <v>26</v>
@@ -6839,17 +6832,17 @@
       </c>
       <c r="L96" s="2"/>
       <c r="M96" s="5" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="N96" s="5" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="O96" s="2"/>
       <c r="P96" s="2"/>
     </row>
     <row r="97" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="B97" s="2"/>
       <c r="C97" s="2" t="s">
@@ -6875,7 +6868,7 @@
     </row>
     <row r="98" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="B98" s="2"/>
       <c r="C98" s="2" t="s">
@@ -6901,7 +6894,7 @@
     </row>
     <row r="99" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="B99" s="2"/>
       <c r="C99" s="2" t="s">

</xml_diff>

<commit_message>
Update map regions and observations
</commit_message>
<xml_diff>
--- a/data/postes_d3s.xlsx
+++ b/data/postes_d3s.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olivierllinares/Documents/01_D3S 2025 2026/DNA 2025 2026/ED3S_Carte_V3_transfert_collegue-2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB84316F-0751-5A48-8113-17B2FA4240D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D27710A2-9702-314C-A38C-AA1518D86343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -147,7 +147,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1174" uniqueCount="663">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="663">
   <si>
     <t>Actif ?</t>
   </si>
@@ -371,9 +371,6 @@
     <t>10000438</t>
   </si>
   <si>
-    <t>AURA</t>
-  </si>
-  <si>
     <t>Saint Trivier de Courtes</t>
   </si>
   <si>
@@ -401,9 +398,6 @@
     <t>EHPAD La Résidence de l'Ourcq à La Ferté-Milon, EHPAD de l'Hôtel Dieu à Oulchy le Château et EHPAD Résidence le Grand Bosquet à Villers-Cotterêts</t>
   </si>
   <si>
-    <t>HdF</t>
-  </si>
-  <si>
     <t xml:space="preserve">49.187787435427694  </t>
   </si>
   <si>
@@ -483,9 +477,6 @@
   </si>
   <si>
     <t>Cagnes-sur-Mer, Vence</t>
-  </si>
-  <si>
-    <t>PACA</t>
   </si>
   <si>
     <t xml:space="preserve">43.66462125670913 </t>
@@ -2137,6 +2128,15 @@
   </si>
   <si>
     <t>6.463718909248732</t>
+  </si>
+  <si>
+    <t>Fléché E Wronski</t>
+  </si>
+  <si>
+    <t>Provence Alpes Cote d'Azur Corse</t>
+  </si>
+  <si>
+    <t>Hauts de France</t>
   </si>
 </sst>
 </file>
@@ -2654,16 +2654,16 @@
         <v>69</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>73</v>
@@ -2689,28 +2689,28 @@
         <v>16</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J3" s="4">
         <v>46258</v>
@@ -2720,10 +2720,10 @@
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="N3" s="5" t="s">
         <v>78</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>79</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
@@ -2733,28 +2733,28 @@
         <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J4" s="4">
         <v>46258</v>
@@ -2764,10 +2764,10 @@
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="N4" s="5" t="s">
         <v>78</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>79</v>
       </c>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
@@ -2783,22 +2783,22 @@
         <v>70</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>51</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="J5" s="4">
         <v>46258</v>
@@ -2808,10 +2808,10 @@
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
@@ -2821,28 +2821,28 @@
         <v>16</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>51</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J6" s="4">
         <v>46258</v>
@@ -2852,10 +2852,10 @@
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
@@ -2865,28 +2865,28 @@
         <v>16</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>101</v>
-      </c>
       <c r="F7" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>51</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J7" s="4">
         <v>46258</v>
@@ -2895,13 +2895,13 @@
         <v>46</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
@@ -2917,19 +2917,19 @@
         <v>70</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="F8" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="4">
@@ -2940,10 +2940,10 @@
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
@@ -2959,22 +2959,22 @@
         <v>70</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H9" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>112</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>115</v>
       </c>
       <c r="J9" s="4">
         <v>46258</v>
@@ -2984,10 +2984,10 @@
       </c>
       <c r="L9" s="2"/>
       <c r="M9" s="5" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="O9" s="2"/>
       <c r="P9" s="2"/>
@@ -2997,16 +2997,16 @@
         <v>16</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>66</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>67</v>
@@ -3018,7 +3018,7 @@
         <v>30</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="J10" s="4">
         <v>46258</v>
@@ -3027,13 +3027,13 @@
         <v>49</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="O10" s="2"/>
       <c r="P10" s="2"/>
@@ -3043,19 +3043,19 @@
         <v>16</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>125</v>
-      </c>
       <c r="F11" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>42</v>
@@ -3064,7 +3064,7 @@
         <v>31</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="J11" s="4">
         <v>46258</v>
@@ -3074,10 +3074,10 @@
       </c>
       <c r="L11" s="2"/>
       <c r="M11" s="5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
@@ -3093,22 +3093,22 @@
         <v>70</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>39</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>112</v>
+        <v>661</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="J12" s="4">
         <v>46258</v>
@@ -3118,10 +3118,10 @@
       </c>
       <c r="L12" s="2"/>
       <c r="M12" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
@@ -3131,19 +3131,19 @@
         <v>16</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>45</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>55</v>
@@ -3152,7 +3152,7 @@
         <v>24</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="J13" s="4">
         <v>46258</v>
@@ -3162,10 +3162,10 @@
       </c>
       <c r="L13" s="2"/>
       <c r="M13" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" s="2"/>
@@ -3175,19 +3175,19 @@
         <v>16</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>45</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>50</v>
@@ -3196,7 +3196,7 @@
         <v>24</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="J14" s="4">
         <v>46258</v>
@@ -3206,10 +3206,10 @@
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="5" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="O14" s="2"/>
       <c r="P14" s="2"/>
@@ -3219,28 +3219,28 @@
         <v>16</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="J15" s="4">
         <v>46258</v>
@@ -3249,13 +3249,13 @@
         <v>46</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="O15" s="2"/>
       <c r="P15" s="2"/>
@@ -3265,19 +3265,19 @@
         <v>16</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D16" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>157</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>34</v>
@@ -3286,7 +3286,7 @@
         <v>24</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="J16" s="4">
         <v>46258</v>
@@ -3296,10 +3296,10 @@
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="5" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="N16" s="5" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="O16" s="2"/>
       <c r="P16" s="2"/>
@@ -3315,13 +3315,13 @@
         <v>70</v>
       </c>
       <c r="D17" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>163</v>
-      </c>
       <c r="F17" s="2" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>34</v>
@@ -3340,10 +3340,10 @@
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" s="2"/>
@@ -3353,19 +3353,19 @@
         <v>16</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>34</v>
@@ -3374,7 +3374,7 @@
         <v>24</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="J18" s="4">
         <v>46258</v>
@@ -3384,10 +3384,10 @@
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="5" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="N18" s="5" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" s="2"/>
@@ -3397,19 +3397,19 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>23</v>
@@ -3418,7 +3418,7 @@
         <v>24</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="J19" s="4">
         <v>46258</v>
@@ -3428,10 +3428,10 @@
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="N19" s="5" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="O19" s="2"/>
       <c r="P19" s="2"/>
@@ -3447,13 +3447,13 @@
         <v>70</v>
       </c>
       <c r="D20" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>178</v>
-      </c>
       <c r="F20" s="2" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>23</v>
@@ -3462,7 +3462,7 @@
         <v>24</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J20" s="4">
         <v>46258</v>
@@ -3472,10 +3472,10 @@
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="5" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="N20" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" s="2"/>
@@ -3491,13 +3491,13 @@
         <v>70</v>
       </c>
       <c r="D21" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>183</v>
-      </c>
       <c r="F21" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>23</v>
@@ -3506,7 +3506,7 @@
         <v>24</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="J21" s="4">
         <v>46258</v>
@@ -3516,10 +3516,10 @@
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="5" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="N21" s="5" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
@@ -3535,13 +3535,13 @@
         <v>70</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>23</v>
@@ -3550,7 +3550,7 @@
         <v>24</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="J22" s="4">
         <v>46258</v>
@@ -3560,10 +3560,10 @@
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="5" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="N22" s="5" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="O22" s="2"/>
       <c r="P22" s="2"/>
@@ -3573,19 +3573,19 @@
         <v>16</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>36</v>
@@ -3594,7 +3594,7 @@
         <v>32</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="J23" s="4">
         <v>46258</v>
@@ -3604,10 +3604,10 @@
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="5" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="N23" s="5" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
@@ -3623,13 +3623,13 @@
         <v>70</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>36</v>
@@ -3638,7 +3638,7 @@
         <v>32</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="J24" s="4">
         <v>46258</v>
@@ -3648,10 +3648,10 @@
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="5" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="N24" s="5" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="O24" s="2"/>
       <c r="P24" s="2"/>
@@ -3667,13 +3667,13 @@
         <v>70</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>36</v>
@@ -3682,7 +3682,7 @@
         <v>32</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="J25" s="4">
         <v>46258</v>
@@ -3692,10 +3692,10 @@
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="5" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="N25" s="5" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="O25" s="2"/>
       <c r="P25" s="2"/>
@@ -3705,28 +3705,28 @@
         <v>16</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="J26" s="4">
         <v>46258</v>
@@ -3736,10 +3736,10 @@
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="5" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="N26" s="5" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="O26" s="2"/>
       <c r="P26" s="2"/>
@@ -3749,19 +3749,19 @@
         <v>16</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D27" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>217</v>
-      </c>
       <c r="F27" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>44</v>
@@ -3780,10 +3780,10 @@
       </c>
       <c r="L27" s="2"/>
       <c r="M27" s="5" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="N27" s="5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="O27" s="2"/>
       <c r="P27" s="2"/>
@@ -3799,22 +3799,22 @@
         <v>70</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="J28" s="4">
         <v>46258</v>
@@ -3824,10 +3824,10 @@
       </c>
       <c r="L28" s="2"/>
       <c r="M28" s="5" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="N28" s="5" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" s="2"/>
@@ -3843,16 +3843,16 @@
         <v>70</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>28</v>
@@ -3866,10 +3866,10 @@
       </c>
       <c r="L29" s="2"/>
       <c r="M29" s="5" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="N29" s="5" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" s="2"/>
@@ -3885,12 +3885,12 @@
         <v>70</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
       <c r="G30" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>28</v>
@@ -3904,10 +3904,10 @@
       </c>
       <c r="L30" s="2"/>
       <c r="M30" s="5" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="N30" s="5" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" s="2"/>
@@ -3917,28 +3917,28 @@
         <v>16</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="J31" s="4">
         <v>46258</v>
@@ -3948,10 +3948,10 @@
       </c>
       <c r="L31" s="2"/>
       <c r="M31" s="5" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="N31" s="5" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="O31" s="2"/>
       <c r="P31" s="2"/>
@@ -3961,28 +3961,28 @@
         <v>16</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="J32" s="4">
         <v>46258</v>
@@ -3992,10 +3992,10 @@
       </c>
       <c r="L32" s="2"/>
       <c r="M32" s="5" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="N32" s="5" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
@@ -4011,13 +4011,13 @@
         <v>70</v>
       </c>
       <c r="D33" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>253</v>
-      </c>
       <c r="F33" s="2" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>18</v>
@@ -4026,7 +4026,7 @@
         <v>19</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="J33" s="4">
         <v>46258</v>
@@ -4035,13 +4035,13 @@
         <v>49</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="M33" s="5" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="N33" s="5" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" s="2"/>
@@ -4051,19 +4051,19 @@
         <v>16</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>257</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>260</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>18</v>
@@ -4072,7 +4072,7 @@
         <v>19</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="J34" s="4">
         <v>46258</v>
@@ -4082,10 +4082,10 @@
       </c>
       <c r="L34" s="2"/>
       <c r="M34" s="5" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="N34" s="5" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="O34" s="2"/>
       <c r="P34" s="2"/>
@@ -4095,19 +4095,19 @@
         <v>16</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>18</v>
@@ -4116,7 +4116,7 @@
         <v>19</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="J35" s="4">
         <v>46258</v>
@@ -4126,10 +4126,10 @@
       </c>
       <c r="L35" s="2"/>
       <c r="M35" s="5" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="N35" s="5" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
@@ -4139,19 +4139,19 @@
         <v>16</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>40</v>
@@ -4160,7 +4160,7 @@
         <v>28</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="J36" s="4">
         <v>46258</v>
@@ -4170,10 +4170,10 @@
       </c>
       <c r="L36" s="2"/>
       <c r="M36" s="5" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="N36" s="5" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
@@ -4183,19 +4183,19 @@
         <v>16</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>47</v>
@@ -4204,7 +4204,7 @@
         <v>28</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="J37" s="4">
         <v>46258</v>
@@ -4214,10 +4214,10 @@
       </c>
       <c r="L37" s="2"/>
       <c r="M37" s="5" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="N37" s="5" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" s="2"/>
@@ -4227,28 +4227,28 @@
         <v>16</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="J38" s="4">
         <v>46258</v>
@@ -4258,10 +4258,10 @@
       </c>
       <c r="L38" s="2"/>
       <c r="M38" s="5" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="N38" s="5" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" s="2"/>
@@ -4271,19 +4271,19 @@
         <v>16</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>54</v>
@@ -4300,10 +4300,10 @@
       </c>
       <c r="L39" s="2"/>
       <c r="M39" s="5" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="N39" s="5" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="O39" s="2"/>
       <c r="P39" s="2"/>
@@ -4319,22 +4319,22 @@
         <v>70</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>24</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="J40" s="4">
         <v>46258</v>
@@ -4344,10 +4344,10 @@
       </c>
       <c r="L40" s="2"/>
       <c r="M40" s="5" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="N40" s="5" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="O40" s="2"/>
       <c r="P40" s="2"/>
@@ -4357,28 +4357,28 @@
         <v>16</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="J41" s="4">
         <v>46258</v>
@@ -4387,13 +4387,13 @@
         <v>49</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="M41" s="5" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="N41" s="5" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>
@@ -4403,28 +4403,28 @@
         <v>16</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="E42" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="F42" s="2" t="s">
-        <v>314</v>
-      </c>
       <c r="G42" s="2" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="J42" s="4">
         <v>46258</v>
@@ -4434,10 +4434,10 @@
       </c>
       <c r="L42" s="2"/>
       <c r="M42" s="5" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="N42" s="5" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="O42" s="2"/>
       <c r="P42" s="2"/>
@@ -4453,22 +4453,22 @@
         <v>70</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="E43" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>319</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>322</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>43</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="J43" s="4">
         <v>46258</v>
@@ -4478,10 +4478,10 @@
       </c>
       <c r="L43" s="2"/>
       <c r="M43" s="5" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="N43" s="5" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="O43" s="2"/>
       <c r="P43" s="2"/>
@@ -4491,28 +4491,28 @@
         <v>16</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E44" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>329</v>
-      </c>
       <c r="F44" s="2" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>31</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="J44" s="4">
         <v>46258</v>
@@ -4522,10 +4522,10 @@
       </c>
       <c r="L44" s="2"/>
       <c r="M44" s="5" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="N44" s="5" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="O44" s="2"/>
       <c r="P44" s="2"/>
@@ -4535,19 +4535,19 @@
         <v>16</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>62</v>
@@ -4556,7 +4556,7 @@
         <v>31</v>
       </c>
       <c r="I45" s="3" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="J45" s="4">
         <v>46258</v>
@@ -4566,10 +4566,10 @@
       </c>
       <c r="L45" s="2"/>
       <c r="M45" s="5" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="N45" s="5" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="O45" s="2"/>
       <c r="P45" s="2"/>
@@ -4579,19 +4579,19 @@
         <v>16</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>62</v>
@@ -4600,7 +4600,7 @@
         <v>31</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="J46" s="4">
         <v>46258</v>
@@ -4610,10 +4610,10 @@
       </c>
       <c r="L46" s="2"/>
       <c r="M46" s="5" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="N46" s="5" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" s="2"/>
@@ -4623,28 +4623,28 @@
         <v>16</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="J47" s="4">
         <v>46258</v>
@@ -4653,13 +4653,13 @@
         <v>49</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="M47" s="5" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="N47" s="5" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
@@ -4669,28 +4669,28 @@
         <v>16</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="J48" s="4">
         <v>46258</v>
@@ -4700,10 +4700,10 @@
       </c>
       <c r="L48" s="2"/>
       <c r="M48" s="5" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="N48" s="5" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" s="2"/>
@@ -4713,28 +4713,28 @@
         <v>16</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="J49" s="4">
         <v>46258</v>
@@ -4744,10 +4744,10 @@
       </c>
       <c r="L49" s="2"/>
       <c r="M49" s="5" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="N49" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="O49" s="2"/>
       <c r="P49" s="2"/>
@@ -4757,28 +4757,28 @@
         <v>16</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="E50" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="F50" s="2" t="s">
         <v>364</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>367</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="J50" s="4">
         <v>46258</v>
@@ -4788,10 +4788,10 @@
       </c>
       <c r="L50" s="2"/>
       <c r="M50" s="5" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="N50" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
@@ -4801,28 +4801,28 @@
         <v>16</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="J51" s="4">
         <v>46258</v>
@@ -4832,10 +4832,10 @@
       </c>
       <c r="L51" s="2"/>
       <c r="M51" s="5" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="N51" s="5" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="O51" s="2"/>
       <c r="P51" s="2"/>
@@ -4845,28 +4845,28 @@
         <v>16</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D52" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>376</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>379</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>58</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="J52" s="4">
         <v>46258</v>
@@ -4876,10 +4876,10 @@
       </c>
       <c r="L52" s="2"/>
       <c r="M52" s="5" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="N52" s="5" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="O52" s="2"/>
       <c r="P52" s="2"/>
@@ -4889,28 +4889,28 @@
         <v>16</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>58</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="J53" s="4">
         <v>46258</v>
@@ -4920,10 +4920,10 @@
       </c>
       <c r="L53" s="2"/>
       <c r="M53" s="5" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="N53" s="5" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="O53" s="2"/>
       <c r="P53" s="2"/>
@@ -4933,28 +4933,28 @@
         <v>16</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D54" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="F54" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="E54" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>394</v>
-      </c>
       <c r="G54" s="2" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="J54" s="4">
         <v>46258</v>
@@ -4963,13 +4963,13 @@
         <v>49</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="N54" s="5" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="O54" s="2"/>
       <c r="P54" s="2"/>
@@ -4985,22 +4985,22 @@
         <v>70</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="J55" s="4">
         <v>46258</v>
@@ -5010,10 +5010,10 @@
       </c>
       <c r="L55" s="2"/>
       <c r="M55" s="5" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="N55" s="5" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="O55" s="2"/>
       <c r="P55" s="2"/>
@@ -5023,28 +5023,28 @@
         <v>16</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>24</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="J56" s="4">
         <v>46258</v>
@@ -5053,13 +5053,13 @@
         <v>49</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="M56" s="5" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="N56" s="5" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="O56" s="2"/>
       <c r="P56" s="2"/>
@@ -5069,28 +5069,28 @@
         <v>16</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>24</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="J57" s="4">
         <v>46258</v>
@@ -5099,13 +5099,13 @@
         <v>49</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="M57" s="5" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="N57" s="5" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="O57" s="2"/>
       <c r="P57" s="2"/>
@@ -5115,19 +5115,19 @@
         <v>16</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>59</v>
@@ -5136,7 +5136,7 @@
         <v>31</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="J58" s="4">
         <v>46258</v>
@@ -5146,10 +5146,10 @@
       </c>
       <c r="L58" s="2"/>
       <c r="M58" s="5" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="N58" s="5" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="O58" s="2"/>
       <c r="P58" s="2"/>
@@ -5165,13 +5165,13 @@
         <v>70</v>
       </c>
       <c r="D59" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="E59" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="E59" s="2" t="s">
-        <v>430</v>
-      </c>
       <c r="F59" s="2" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>59</v>
@@ -5180,7 +5180,7 @@
         <v>31</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="J59" s="4">
         <v>46258</v>
@@ -5190,10 +5190,10 @@
       </c>
       <c r="L59" s="2"/>
       <c r="M59" s="5" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="N59" s="5" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="O59" s="2"/>
       <c r="P59" s="2"/>
@@ -5203,19 +5203,19 @@
         <v>16</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>59</v>
@@ -5224,7 +5224,7 @@
         <v>31</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="J60" s="4">
         <v>46258</v>
@@ -5234,10 +5234,10 @@
       </c>
       <c r="L60" s="2"/>
       <c r="M60" s="5" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="N60" s="5" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="O60" s="2"/>
       <c r="P60" s="2"/>
@@ -5247,19 +5247,19 @@
         <v>16</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>59</v>
@@ -5268,7 +5268,7 @@
         <v>31</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="J61" s="4">
         <v>46258</v>
@@ -5277,13 +5277,13 @@
         <v>49</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="M61" s="5" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="N61" s="5" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" s="2"/>
@@ -5296,16 +5296,16 @@
         <v>17</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D62" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E62" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="E62" s="2" t="s">
-        <v>449</v>
-      </c>
       <c r="F62" s="2" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>59</v>
@@ -5314,7 +5314,7 @@
         <v>31</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="J62" s="4">
         <v>46258</v>
@@ -5324,10 +5324,10 @@
       </c>
       <c r="L62" s="2"/>
       <c r="M62" s="5" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="N62" s="5" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="O62" s="2"/>
       <c r="P62" s="2"/>
@@ -5337,19 +5337,19 @@
         <v>16</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>33</v>
@@ -5358,7 +5358,7 @@
         <v>31</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="J63" s="4">
         <v>46258</v>
@@ -5367,13 +5367,13 @@
         <v>49</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="M63" s="5" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="N63" s="5" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="O63" s="2"/>
       <c r="P63" s="2"/>
@@ -5383,19 +5383,19 @@
         <v>16</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>33</v>
@@ -5404,7 +5404,7 @@
         <v>31</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="J64" s="4">
         <v>46258</v>
@@ -5414,10 +5414,10 @@
       </c>
       <c r="L64" s="2"/>
       <c r="M64" s="5" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="N64" s="5" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="O64" s="2"/>
       <c r="P64" s="2"/>
@@ -5433,22 +5433,22 @@
         <v>70</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="H65" s="2" t="s">
         <v>32</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="J65" s="4">
         <v>46258</v>
@@ -5458,10 +5458,10 @@
       </c>
       <c r="L65" s="2"/>
       <c r="M65" s="5" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="N65" s="5" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
@@ -5471,28 +5471,28 @@
         <v>16</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>32</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="J66" s="4">
         <v>46258</v>
@@ -5502,10 +5502,10 @@
       </c>
       <c r="L66" s="2"/>
       <c r="M66" s="5" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="N66" s="5" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="O66" s="2"/>
       <c r="P66" s="2"/>
@@ -5521,22 +5521,22 @@
         <v>70</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="H67" s="2" t="s">
         <v>32</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="J67" s="4">
         <v>46258</v>
@@ -5546,10 +5546,10 @@
       </c>
       <c r="L67" s="2"/>
       <c r="M67" s="5" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="N67" s="5" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="O67" s="2"/>
       <c r="P67" s="2"/>
@@ -5559,28 +5559,28 @@
         <v>16</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="I68" s="3" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="J68" s="4">
         <v>46258</v>
@@ -5590,10 +5590,10 @@
       </c>
       <c r="L68" s="2"/>
       <c r="M68" s="5" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="N68" s="5" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="O68" s="2"/>
       <c r="P68" s="2"/>
@@ -5609,22 +5609,22 @@
         <v>70</v>
       </c>
       <c r="D69" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="E69" s="2" t="s">
         <v>487</v>
       </c>
-      <c r="E69" s="2" t="s">
-        <v>490</v>
-      </c>
       <c r="F69" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="J69" s="4">
         <v>46258</v>
@@ -5634,10 +5634,10 @@
       </c>
       <c r="L69" s="2"/>
       <c r="M69" s="5" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="N69" s="5" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="O69" s="2"/>
       <c r="P69" s="2"/>
@@ -5647,28 +5647,28 @@
         <v>16</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="J70" s="4">
         <v>46258</v>
@@ -5677,13 +5677,13 @@
         <v>49</v>
       </c>
       <c r="L70" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="M70" s="5" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="N70" s="5" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="O70" s="2"/>
       <c r="P70" s="2"/>
@@ -5693,22 +5693,22 @@
         <v>16</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>22</v>
@@ -5721,13 +5721,13 @@
         <v>49</v>
       </c>
       <c r="L71" s="2" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="M71" s="5" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="N71" s="5" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="O71" s="2"/>
       <c r="P71" s="2"/>
@@ -5737,28 +5737,28 @@
         <v>16</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>41</v>
       </c>
       <c r="I72" s="3" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="J72" s="4">
         <v>46258</v>
@@ -5767,13 +5767,13 @@
         <v>49</v>
       </c>
       <c r="L72" s="2" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="M72" s="5" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="N72" s="5" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="O72" s="2"/>
       <c r="P72" s="2"/>
@@ -5783,28 +5783,28 @@
         <v>16</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>41</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="J73" s="4">
         <v>46258</v>
@@ -5814,10 +5814,10 @@
       </c>
       <c r="L73" s="2"/>
       <c r="M73" s="5" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="N73" s="5" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="O73" s="2"/>
       <c r="P73" s="2"/>
@@ -5827,28 +5827,28 @@
         <v>16</v>
       </c>
       <c r="B74" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="E74" s="2" t="s">
         <v>523</v>
       </c>
-      <c r="C74" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>522</v>
-      </c>
-      <c r="E74" s="2" t="s">
-        <v>526</v>
-      </c>
       <c r="F74" s="2" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="J74" s="4">
         <v>46258</v>
@@ -5858,10 +5858,10 @@
       </c>
       <c r="L74" s="2"/>
       <c r="M74" s="5" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="N74" s="5" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="O74" s="2"/>
       <c r="P74" s="2"/>
@@ -5871,28 +5871,28 @@
         <v>16</v>
       </c>
       <c r="B75" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="F75" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="C75" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>528</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="F75" s="2" t="s">
-        <v>532</v>
-      </c>
       <c r="G75" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="J75" s="4">
         <v>46258</v>
@@ -5902,10 +5902,10 @@
       </c>
       <c r="L75" s="2"/>
       <c r="M75" s="5" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="N75" s="5" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="O75" s="2"/>
       <c r="P75" s="2"/>
@@ -5915,28 +5915,28 @@
         <v>16</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="J76" s="4">
         <v>46258</v>
@@ -5945,13 +5945,13 @@
         <v>49</v>
       </c>
       <c r="L76" s="2" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="M76" s="5" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="N76" s="5" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="O76" s="2"/>
       <c r="P76" s="2"/>
@@ -5964,22 +5964,22 @@
         <v>17</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D77" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="E77" s="2" t="s">
         <v>541</v>
       </c>
-      <c r="E77" s="2" t="s">
-        <v>544</v>
-      </c>
       <c r="F77" s="2" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="I77" s="3"/>
       <c r="J77" s="4">
@@ -5990,10 +5990,10 @@
       </c>
       <c r="L77" s="2"/>
       <c r="M77" s="5" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="N77" s="5" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="O77" s="2"/>
       <c r="P77" s="2"/>
@@ -6003,28 +6003,28 @@
         <v>16</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D78" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="F78" s="2" t="s">
         <v>547</v>
       </c>
-      <c r="E78" s="2" t="s">
-        <v>549</v>
-      </c>
-      <c r="F78" s="2" t="s">
-        <v>550</v>
-      </c>
       <c r="G78" s="2" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="J78" s="4">
         <v>46258</v>
@@ -6034,10 +6034,10 @@
       </c>
       <c r="L78" s="2"/>
       <c r="M78" s="5" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="N78" s="5" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="O78" s="2"/>
       <c r="P78" s="2"/>
@@ -6047,19 +6047,19 @@
         <v>16</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="G79" s="2" t="s">
         <v>25</v>
@@ -6068,7 +6068,7 @@
         <v>24</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="J79" s="4">
         <v>46258</v>
@@ -6078,10 +6078,10 @@
       </c>
       <c r="L79" s="2"/>
       <c r="M79" s="5" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="N79" s="5" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="O79" s="2"/>
       <c r="P79" s="2"/>
@@ -6091,16 +6091,16 @@
         <v>16</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>52</v>
@@ -6109,10 +6109,10 @@
         <v>53</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>84</v>
+        <v>662</v>
       </c>
       <c r="I80" s="3" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="J80" s="4">
         <v>46258</v>
@@ -6121,13 +6121,13 @@
         <v>49</v>
       </c>
       <c r="L80" s="2" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="M80" s="5" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="N80" s="5" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="O80" s="2"/>
       <c r="P80" s="2"/>
@@ -6137,25 +6137,25 @@
         <v>16</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="G81" s="2" t="s">
         <v>29</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>112</v>
+        <v>661</v>
       </c>
       <c r="I81" s="3"/>
       <c r="J81" s="4">
@@ -6166,10 +6166,10 @@
       </c>
       <c r="L81" s="2"/>
       <c r="M81" s="5" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="N81" s="5" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="O81" s="2"/>
       <c r="P81" s="2"/>
@@ -6179,25 +6179,25 @@
         <v>16</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="G82" s="2" t="s">
         <v>29</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>112</v>
+        <v>661</v>
       </c>
       <c r="I82" s="3"/>
       <c r="J82" s="4">
@@ -6208,10 +6208,10 @@
       </c>
       <c r="L82" s="2"/>
       <c r="M82" s="5" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="N82" s="5" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="O82" s="2"/>
       <c r="P82" s="2"/>
@@ -6221,28 +6221,28 @@
         <v>16</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="H83" s="2" t="s">
         <v>24</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="J83" s="4">
         <v>46258</v>
@@ -6252,10 +6252,10 @@
       </c>
       <c r="L83" s="2"/>
       <c r="M83" s="5" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="N83" s="5" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="O83" s="2"/>
       <c r="P83" s="2"/>
@@ -6265,19 +6265,19 @@
         <v>16</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="G84" s="2" t="s">
         <v>38</v>
@@ -6286,7 +6286,7 @@
         <v>24</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="J84" s="4">
         <v>46258</v>
@@ -6296,10 +6296,10 @@
       </c>
       <c r="L84" s="2"/>
       <c r="M84" s="5" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="N84" s="5" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="O84" s="2"/>
       <c r="P84" s="2"/>
@@ -6315,13 +6315,13 @@
         <v>70</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>38</v>
@@ -6330,7 +6330,7 @@
         <v>24</v>
       </c>
       <c r="I85" s="3" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="J85" s="4">
         <v>46258</v>
@@ -6340,10 +6340,10 @@
       </c>
       <c r="L85" s="2"/>
       <c r="M85" s="5" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="N85" s="5" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="O85" s="2"/>
       <c r="P85" s="2"/>
@@ -6359,13 +6359,13 @@
         <v>70</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="G86" s="2" t="s">
         <v>38</v>
@@ -6374,7 +6374,7 @@
         <v>24</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="J86" s="4">
         <v>46258</v>
@@ -6384,10 +6384,10 @@
       </c>
       <c r="L86" s="2"/>
       <c r="M86" s="5" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="N86" s="5" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="O86" s="2"/>
       <c r="P86" s="2"/>
@@ -6397,19 +6397,19 @@
         <v>16</v>
       </c>
       <c r="B87" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="F87" s="2" t="s">
         <v>589</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>588</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>591</v>
-      </c>
-      <c r="F87" s="2" t="s">
-        <v>592</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>37</v>
@@ -6418,7 +6418,7 @@
         <v>32</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="J87" s="4">
         <v>46258</v>
@@ -6427,13 +6427,13 @@
         <v>49</v>
       </c>
       <c r="L87" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="M87" s="5" t="s">
         <v>590</v>
       </c>
-      <c r="M87" s="5" t="s">
-        <v>593</v>
-      </c>
       <c r="N87" s="5" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="O87" s="2"/>
       <c r="P87" s="2"/>
@@ -6443,19 +6443,19 @@
         <v>16</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>37</v>
@@ -6464,7 +6464,7 @@
         <v>32</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="J88" s="4">
         <v>46258</v>
@@ -6474,10 +6474,10 @@
       </c>
       <c r="L88" s="2"/>
       <c r="M88" s="5" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="N88" s="5" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="O88" s="2"/>
       <c r="P88" s="2"/>
@@ -6487,28 +6487,28 @@
         <v>16</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="H89" s="2" t="s">
         <v>32</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="J89" s="4">
         <v>46258</v>
@@ -6518,10 +6518,10 @@
       </c>
       <c r="L89" s="2"/>
       <c r="M89" s="5" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="N89" s="5" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="O89" s="2"/>
       <c r="P89" s="2"/>
@@ -6531,28 +6531,28 @@
         <v>16</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>57</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="J90" s="4">
         <v>46258</v>
@@ -6561,13 +6561,13 @@
         <v>49</v>
       </c>
       <c r="L90" s="2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="M90" s="5" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="N90" s="5" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="O90" s="2"/>
       <c r="P90" s="2"/>
@@ -6577,28 +6577,28 @@
         <v>16</v>
       </c>
       <c r="B91" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="E91" s="2" t="s">
         <v>618</v>
       </c>
-      <c r="C91" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D91" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="E91" s="2" t="s">
-        <v>621</v>
-      </c>
       <c r="F91" s="2" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>57</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="J91" s="4">
         <v>46258</v>
@@ -6608,10 +6608,10 @@
       </c>
       <c r="L91" s="2"/>
       <c r="M91" s="5" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="N91" s="5" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="O91" s="2"/>
       <c r="P91" s="2"/>
@@ -6621,28 +6621,28 @@
         <v>16</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D92" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="E92" s="2" t="s">
         <v>623</v>
       </c>
-      <c r="E92" s="2" t="s">
-        <v>626</v>
-      </c>
       <c r="F92" s="2" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="G92" s="2" t="s">
         <v>57</v>
       </c>
       <c r="H92" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="J92" s="4">
         <v>46258</v>
@@ -6651,13 +6651,13 @@
         <v>49</v>
       </c>
       <c r="L92" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="M92" s="5" t="s">
+        <v>624</v>
+      </c>
+      <c r="N92" s="5" t="s">
         <v>625</v>
-      </c>
-      <c r="M92" s="5" t="s">
-        <v>627</v>
-      </c>
-      <c r="N92" s="5" t="s">
-        <v>628</v>
       </c>
       <c r="O92" s="2"/>
       <c r="P92" s="2"/>
@@ -6667,28 +6667,28 @@
         <v>16</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>57</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="I93" s="3" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="J93" s="4">
         <v>46258</v>
@@ -6698,10 +6698,10 @@
       </c>
       <c r="L93" s="2"/>
       <c r="M93" s="5" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="N93" s="5" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="O93" s="2"/>
       <c r="P93" s="2"/>
@@ -6711,28 +6711,28 @@
         <v>16</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D94" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="G94" s="2" t="s">
         <v>636</v>
       </c>
-      <c r="E94" s="2" t="s">
-        <v>638</v>
-      </c>
-      <c r="F94" s="2" t="s">
-        <v>638</v>
-      </c>
-      <c r="G94" s="2" t="s">
-        <v>639</v>
-      </c>
       <c r="H94" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="I94" s="3" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="J94" s="4">
         <v>46258</v>
@@ -6741,13 +6741,13 @@
         <v>49</v>
       </c>
       <c r="L94" s="2" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="M94" s="5" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="N94" s="5" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="O94" s="2"/>
       <c r="P94" s="2"/>
@@ -6757,28 +6757,28 @@
         <v>16</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="I95" s="3" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="J95" s="4">
         <v>46258</v>
@@ -6787,13 +6787,13 @@
         <v>60</v>
       </c>
       <c r="L95" s="2" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="M95" s="5" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="N95" s="5" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="O95" s="2"/>
       <c r="P95" s="2"/>
@@ -6803,19 +6803,19 @@
         <v>16</v>
       </c>
       <c r="B96" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="E96" s="2" t="s">
         <v>651</v>
       </c>
-      <c r="C96" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D96" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="E96" s="2" t="s">
-        <v>654</v>
-      </c>
       <c r="F96" s="2" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="G96" s="2" t="s">
         <v>26</v>
@@ -6830,19 +6830,21 @@
       <c r="K96" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="L96" s="2"/>
+      <c r="L96" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M96" s="5" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="N96" s="5" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="O96" s="2"/>
       <c r="P96" s="2"/>
     </row>
     <row r="97" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="B97" s="2"/>
       <c r="C97" s="2" t="s">
@@ -6868,7 +6870,7 @@
     </row>
     <row r="98" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="B98" s="2"/>
       <c r="C98" s="2" t="s">
@@ -6894,7 +6896,7 @@
     </row>
     <row r="99" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="B99" s="2"/>
       <c r="C99" s="2" t="s">

</xml_diff>

<commit_message>
Update post availability and Grand-Fougeray location
</commit_message>
<xml_diff>
--- a/data/postes_d3s.xlsx
+++ b/data/postes_d3s.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olivierllinares/Documents/01_D3S 2025 2026/DNA 2025 2026/ED3S_Carte_V3_transfert_collegue-2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D27710A2-9702-314C-A38C-AA1518D86343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45EDD17B-3E3B-6D4C-94AE-75949F14639B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -147,7 +147,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="663">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1247" uniqueCount="663">
   <si>
     <t>Actif ?</t>
   </si>
@@ -887,16 +887,7 @@
     <t>Directeur adjoint du FDEF</t>
   </si>
   <si>
-    <t>350058376</t>
-  </si>
-  <si>
     <t>EPSMS Les Horizons au Grand-Fougeray</t>
-  </si>
-  <si>
-    <t>47.72556530979014 -</t>
-  </si>
-  <si>
-    <t>1.7330950850567624</t>
   </si>
   <si>
     <t>Grand-Fougeray</t>
@@ -2137,6 +2128,15 @@
   </si>
   <si>
     <t>Hauts de France</t>
+  </si>
+  <si>
+    <t>Ouvert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47.72556530979014 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -1.7330950850567624</t>
   </si>
 </sst>
 </file>
@@ -2674,7 +2674,9 @@
       <c r="K2" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L2" s="2"/>
+      <c r="L2" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M2" s="5" t="s">
         <v>72</v>
       </c>
@@ -2718,7 +2720,9 @@
       <c r="K3" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L3" s="2"/>
+      <c r="L3" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M3" s="5" t="s">
         <v>77</v>
       </c>
@@ -2762,7 +2766,9 @@
       <c r="K4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L4" s="2"/>
+      <c r="L4" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M4" s="5" t="s">
         <v>77</v>
       </c>
@@ -2795,7 +2801,7 @@
         <v>51</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>85</v>
@@ -2806,7 +2812,9 @@
       <c r="K5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L5" s="2"/>
+      <c r="L5" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M5" s="5" t="s">
         <v>83</v>
       </c>
@@ -2839,7 +2847,7 @@
         <v>51</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>92</v>
@@ -2850,7 +2858,9 @@
       <c r="K6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L6" s="2"/>
+      <c r="L6" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M6" s="5" t="s">
         <v>94</v>
       </c>
@@ -2883,7 +2893,7 @@
         <v>51</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>102</v>
@@ -2938,7 +2948,9 @@
       <c r="K8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L8" s="2"/>
+      <c r="L8" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M8" s="5" t="s">
         <v>107</v>
       </c>
@@ -2971,7 +2983,7 @@
         <v>109</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>112</v>
@@ -2982,7 +2994,9 @@
       <c r="K9" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L9" s="2"/>
+      <c r="L9" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M9" s="5" t="s">
         <v>110</v>
       </c>
@@ -3072,7 +3086,9 @@
       <c r="K11" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L11" s="2"/>
+      <c r="L11" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M11" s="5" t="s">
         <v>123</v>
       </c>
@@ -3105,7 +3121,7 @@
         <v>39</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>126</v>
@@ -3116,7 +3132,9 @@
       <c r="K12" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L12" s="2"/>
+      <c r="L12" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M12" s="5" t="s">
         <v>129</v>
       </c>
@@ -3160,7 +3178,9 @@
       <c r="K13" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L13" s="2"/>
+      <c r="L13" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M13" s="5" t="s">
         <v>136</v>
       </c>
@@ -3184,10 +3204,10 @@
         <v>139</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>50</v>
@@ -3204,12 +3224,14 @@
       <c r="K14" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L14" s="2"/>
+      <c r="L14" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M14" s="5" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="O14" s="2"/>
       <c r="P14" s="2"/>
@@ -3294,7 +3316,9 @@
       <c r="K16" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L16" s="2"/>
+      <c r="L16" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M16" s="5" t="s">
         <v>155</v>
       </c>
@@ -3338,7 +3362,9 @@
       <c r="K17" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L17" s="2"/>
+      <c r="L17" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M17" s="5" t="s">
         <v>158</v>
       </c>
@@ -3382,7 +3408,9 @@
       <c r="K18" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L18" s="2"/>
+      <c r="L18" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M18" s="5" t="s">
         <v>164</v>
       </c>
@@ -3426,7 +3454,9 @@
       <c r="K19" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L19" s="2"/>
+      <c r="L19" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M19" s="5" t="s">
         <v>169</v>
       </c>
@@ -3470,7 +3500,9 @@
       <c r="K20" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L20" s="2"/>
+      <c r="L20" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M20" s="5" t="s">
         <v>173</v>
       </c>
@@ -3514,7 +3546,9 @@
       <c r="K21" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L21" s="2"/>
+      <c r="L21" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M21" s="5" t="s">
         <v>178</v>
       </c>
@@ -3558,7 +3592,9 @@
       <c r="K22" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L22" s="2"/>
+      <c r="L22" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M22" s="5" t="s">
         <v>182</v>
       </c>
@@ -3602,7 +3638,9 @@
       <c r="K23" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L23" s="2"/>
+      <c r="L23" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M23" s="5" t="s">
         <v>191</v>
       </c>
@@ -3646,7 +3684,9 @@
       <c r="K24" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L24" s="2"/>
+      <c r="L24" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M24" s="5" t="s">
         <v>199</v>
       </c>
@@ -3690,7 +3730,9 @@
       <c r="K25" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L25" s="2"/>
+      <c r="L25" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M25" s="5" t="s">
         <v>201</v>
       </c>
@@ -3734,7 +3776,9 @@
       <c r="K26" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L26" s="2"/>
+      <c r="L26" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M26" s="5" t="s">
         <v>209</v>
       </c>
@@ -3778,7 +3822,9 @@
       <c r="K27" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L27" s="2"/>
+      <c r="L27" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M27" s="5" t="s">
         <v>215</v>
       </c>
@@ -3822,7 +3868,9 @@
       <c r="K28" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L28" s="2"/>
+      <c r="L28" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M28" s="5" t="s">
         <v>222</v>
       </c>
@@ -3864,7 +3912,9 @@
       <c r="K29" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L29" s="2"/>
+      <c r="L29" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M29" s="5" t="s">
         <v>230</v>
       </c>
@@ -3902,7 +3952,9 @@
       <c r="K30" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L30" s="2"/>
+      <c r="L30" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M30" s="5" t="s">
         <v>228</v>
       </c>
@@ -3946,7 +3998,9 @@
       <c r="K31" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L31" s="2"/>
+      <c r="L31" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M31" s="5" t="s">
         <v>237</v>
       </c>
@@ -3990,7 +4044,9 @@
       <c r="K32" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L32" s="2"/>
+      <c r="L32" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M32" s="5" t="s">
         <v>243</v>
       </c>
@@ -4000,7 +4056,7 @@
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
     </row>
-    <row r="33" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>16</v>
       </c>
@@ -4011,13 +4067,13 @@
         <v>70</v>
       </c>
       <c r="D33" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>250</v>
-      </c>
       <c r="F33" s="2" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>18</v>
@@ -4025,9 +4081,7 @@
       <c r="H33" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I33" s="3" t="s">
-        <v>246</v>
-      </c>
+      <c r="I33" s="3"/>
       <c r="J33" s="4">
         <v>46258</v>
       </c>
@@ -4035,13 +4089,13 @@
         <v>49</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="M33" s="5" t="s">
-        <v>248</v>
+        <v>661</v>
       </c>
       <c r="N33" s="5" t="s">
-        <v>249</v>
+        <v>662</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" s="2"/>
@@ -4051,19 +4105,19 @@
         <v>16</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>254</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>257</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>18</v>
@@ -4072,7 +4126,7 @@
         <v>19</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J34" s="4">
         <v>46258</v>
@@ -4080,12 +4134,14 @@
       <c r="K34" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L34" s="2"/>
+      <c r="L34" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M34" s="5" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="N34" s="5" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="O34" s="2"/>
       <c r="P34" s="2"/>
@@ -4095,19 +4151,19 @@
         <v>16</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>18</v>
@@ -4116,7 +4172,7 @@
         <v>19</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="J35" s="4">
         <v>46258</v>
@@ -4124,12 +4180,14 @@
       <c r="K35" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L35" s="2"/>
+      <c r="L35" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M35" s="5" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="N35" s="5" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
@@ -4139,19 +4197,19 @@
         <v>16</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>40</v>
@@ -4160,7 +4218,7 @@
         <v>28</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="J36" s="4">
         <v>46258</v>
@@ -4168,12 +4226,14 @@
       <c r="K36" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L36" s="2"/>
+      <c r="L36" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M36" s="5" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="N36" s="5" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
@@ -4183,19 +4243,19 @@
         <v>16</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>47</v>
@@ -4204,7 +4264,7 @@
         <v>28</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="J37" s="4">
         <v>46258</v>
@@ -4212,12 +4272,14 @@
       <c r="K37" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L37" s="2"/>
+      <c r="L37" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M37" s="5" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="N37" s="5" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" s="2"/>
@@ -4227,28 +4289,28 @@
         <v>16</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="J38" s="4">
         <v>46258</v>
@@ -4256,12 +4318,14 @@
       <c r="K38" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L38" s="2"/>
+      <c r="L38" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M38" s="5" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="N38" s="5" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" s="2"/>
@@ -4271,19 +4335,19 @@
         <v>16</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>54</v>
@@ -4298,12 +4362,14 @@
       <c r="K39" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L39" s="2"/>
+      <c r="L39" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M39" s="5" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="N39" s="5" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="O39" s="2"/>
       <c r="P39" s="2"/>
@@ -4319,22 +4385,22 @@
         <v>70</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>24</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="J40" s="4">
         <v>46258</v>
@@ -4342,12 +4408,14 @@
       <c r="K40" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L40" s="2"/>
+      <c r="L40" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M40" s="5" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="N40" s="5" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="O40" s="2"/>
       <c r="P40" s="2"/>
@@ -4357,28 +4425,28 @@
         <v>16</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="J41" s="4">
         <v>46258</v>
@@ -4387,13 +4455,13 @@
         <v>49</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="M41" s="5" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="N41" s="5" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>
@@ -4403,28 +4471,28 @@
         <v>16</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="E42" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="F42" s="2" t="s">
-        <v>311</v>
-      </c>
       <c r="G42" s="2" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="J42" s="4">
         <v>46258</v>
@@ -4432,12 +4500,14 @@
       <c r="K42" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L42" s="2"/>
+      <c r="L42" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M42" s="5" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="N42" s="5" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="O42" s="2"/>
       <c r="P42" s="2"/>
@@ -4453,22 +4523,22 @@
         <v>70</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="E43" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>316</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>319</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>43</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="J43" s="4">
         <v>46258</v>
@@ -4476,12 +4546,14 @@
       <c r="K43" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L43" s="2"/>
+      <c r="L43" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M43" s="5" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="N43" s="5" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="O43" s="2"/>
       <c r="P43" s="2"/>
@@ -4491,28 +4563,28 @@
         <v>16</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>31</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="J44" s="4">
         <v>46258</v>
@@ -4520,12 +4592,14 @@
       <c r="K44" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L44" s="2"/>
+      <c r="L44" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M44" s="5" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="N44" s="5" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="O44" s="2"/>
       <c r="P44" s="2"/>
@@ -4535,19 +4609,19 @@
         <v>16</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>62</v>
@@ -4556,7 +4630,7 @@
         <v>31</v>
       </c>
       <c r="I45" s="3" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="J45" s="4">
         <v>46258</v>
@@ -4564,12 +4638,14 @@
       <c r="K45" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L45" s="2"/>
+      <c r="L45" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M45" s="5" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="N45" s="5" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="O45" s="2"/>
       <c r="P45" s="2"/>
@@ -4579,19 +4655,19 @@
         <v>16</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>62</v>
@@ -4600,7 +4676,7 @@
         <v>31</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="J46" s="4">
         <v>46258</v>
@@ -4608,12 +4684,14 @@
       <c r="K46" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L46" s="2"/>
+      <c r="L46" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M46" s="5" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="N46" s="5" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" s="2"/>
@@ -4623,28 +4701,28 @@
         <v>16</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="J47" s="4">
         <v>46258</v>
@@ -4653,13 +4731,13 @@
         <v>49</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="M47" s="5" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="N47" s="5" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
@@ -4669,28 +4747,28 @@
         <v>16</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="J48" s="4">
         <v>46258</v>
@@ -4698,12 +4776,14 @@
       <c r="K48" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L48" s="2"/>
+      <c r="L48" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M48" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="N48" s="5" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" s="2"/>
@@ -4719,22 +4799,22 @@
         <v>76</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="J49" s="4">
         <v>46258</v>
@@ -4742,12 +4822,14 @@
       <c r="K49" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L49" s="2"/>
+      <c r="L49" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M49" s="5" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="N49" s="5" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="O49" s="2"/>
       <c r="P49" s="2"/>
@@ -4757,28 +4839,28 @@
         <v>16</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="E50" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="F50" s="2" t="s">
         <v>361</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>364</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="J50" s="4">
         <v>46258</v>
@@ -4786,12 +4868,14 @@
       <c r="K50" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L50" s="2"/>
+      <c r="L50" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M50" s="5" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="N50" s="5" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
@@ -4801,28 +4885,28 @@
         <v>16</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="J51" s="4">
         <v>46258</v>
@@ -4830,12 +4914,14 @@
       <c r="K51" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L51" s="2"/>
+      <c r="L51" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M51" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="N51" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="O51" s="2"/>
       <c r="P51" s="2"/>
@@ -4845,28 +4931,28 @@
         <v>16</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D52" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>373</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>376</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>58</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="J52" s="4">
         <v>46258</v>
@@ -4874,12 +4960,14 @@
       <c r="K52" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L52" s="2"/>
+      <c r="L52" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M52" s="5" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="N52" s="5" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="O52" s="2"/>
       <c r="P52" s="2"/>
@@ -4889,28 +4977,28 @@
         <v>16</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>58</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="J53" s="4">
         <v>46258</v>
@@ -4918,12 +5006,14 @@
       <c r="K53" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L53" s="2"/>
+      <c r="L53" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M53" s="5" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="N53" s="5" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="O53" s="2"/>
       <c r="P53" s="2"/>
@@ -4933,28 +5023,28 @@
         <v>16</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D54" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="F54" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="E54" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>391</v>
-      </c>
       <c r="G54" s="2" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="J54" s="4">
         <v>46258</v>
@@ -4963,13 +5053,13 @@
         <v>49</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="N54" s="5" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="O54" s="2"/>
       <c r="P54" s="2"/>
@@ -4985,22 +5075,22 @@
         <v>70</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="J55" s="4">
         <v>46258</v>
@@ -5008,12 +5098,14 @@
       <c r="K55" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L55" s="2"/>
+      <c r="L55" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M55" s="5" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="N55" s="5" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="O55" s="2"/>
       <c r="P55" s="2"/>
@@ -5023,28 +5115,28 @@
         <v>16</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>24</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="J56" s="4">
         <v>46258</v>
@@ -5053,13 +5145,13 @@
         <v>49</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="M56" s="5" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="N56" s="5" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="O56" s="2"/>
       <c r="P56" s="2"/>
@@ -5069,28 +5161,28 @@
         <v>16</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>24</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="J57" s="4">
         <v>46258</v>
@@ -5099,13 +5191,13 @@
         <v>49</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="M57" s="5" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="N57" s="5" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="O57" s="2"/>
       <c r="P57" s="2"/>
@@ -5115,19 +5207,19 @@
         <v>16</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>59</v>
@@ -5136,7 +5228,7 @@
         <v>31</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="J58" s="4">
         <v>46258</v>
@@ -5144,12 +5236,14 @@
       <c r="K58" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L58" s="2"/>
+      <c r="L58" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M58" s="5" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="N58" s="5" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="O58" s="2"/>
       <c r="P58" s="2"/>
@@ -5165,13 +5259,13 @@
         <v>70</v>
       </c>
       <c r="D59" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E59" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="E59" s="2" t="s">
-        <v>427</v>
-      </c>
       <c r="F59" s="2" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>59</v>
@@ -5180,7 +5274,7 @@
         <v>31</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="J59" s="4">
         <v>46258</v>
@@ -5188,12 +5282,14 @@
       <c r="K59" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L59" s="2"/>
+      <c r="L59" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M59" s="5" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="N59" s="5" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="O59" s="2"/>
       <c r="P59" s="2"/>
@@ -5203,19 +5299,19 @@
         <v>16</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>59</v>
@@ -5224,7 +5320,7 @@
         <v>31</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="J60" s="4">
         <v>46258</v>
@@ -5232,12 +5328,14 @@
       <c r="K60" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L60" s="2"/>
+      <c r="L60" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M60" s="5" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="N60" s="5" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="O60" s="2"/>
       <c r="P60" s="2"/>
@@ -5247,19 +5345,19 @@
         <v>16</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>59</v>
@@ -5268,7 +5366,7 @@
         <v>31</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="J61" s="4">
         <v>46258</v>
@@ -5277,13 +5375,13 @@
         <v>49</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="M61" s="5" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="N61" s="5" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" s="2"/>
@@ -5299,13 +5397,13 @@
         <v>76</v>
       </c>
       <c r="D62" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="E62" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="E62" s="2" t="s">
-        <v>446</v>
-      </c>
       <c r="F62" s="2" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>59</v>
@@ -5314,7 +5412,7 @@
         <v>31</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="J62" s="4">
         <v>46258</v>
@@ -5322,12 +5420,14 @@
       <c r="K62" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L62" s="2"/>
+      <c r="L62" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M62" s="5" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="N62" s="5" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="O62" s="2"/>
       <c r="P62" s="2"/>
@@ -5337,19 +5437,19 @@
         <v>16</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>33</v>
@@ -5358,7 +5458,7 @@
         <v>31</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="J63" s="4">
         <v>46258</v>
@@ -5367,13 +5467,13 @@
         <v>49</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="M63" s="5" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="N63" s="5" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="O63" s="2"/>
       <c r="P63" s="2"/>
@@ -5383,19 +5483,19 @@
         <v>16</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>33</v>
@@ -5404,7 +5504,7 @@
         <v>31</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="J64" s="4">
         <v>46258</v>
@@ -5412,12 +5512,14 @@
       <c r="K64" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L64" s="2"/>
+      <c r="L64" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M64" s="5" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="N64" s="5" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="O64" s="2"/>
       <c r="P64" s="2"/>
@@ -5433,22 +5535,22 @@
         <v>70</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="H65" s="2" t="s">
         <v>32</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="J65" s="4">
         <v>46258</v>
@@ -5456,12 +5558,14 @@
       <c r="K65" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L65" s="2"/>
+      <c r="L65" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M65" s="5" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="N65" s="5" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
@@ -5471,28 +5575,28 @@
         <v>16</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>32</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="J66" s="4">
         <v>46258</v>
@@ -5500,12 +5604,14 @@
       <c r="K66" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L66" s="2"/>
+      <c r="L66" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M66" s="5" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="N66" s="5" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="O66" s="2"/>
       <c r="P66" s="2"/>
@@ -5521,22 +5627,22 @@
         <v>70</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="H67" s="2" t="s">
         <v>32</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="J67" s="4">
         <v>46258</v>
@@ -5544,12 +5650,14 @@
       <c r="K67" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L67" s="2"/>
+      <c r="L67" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M67" s="5" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="N67" s="5" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="O67" s="2"/>
       <c r="P67" s="2"/>
@@ -5559,28 +5667,28 @@
         <v>16</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="C68" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="I68" s="3" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="J68" s="4">
         <v>46258</v>
@@ -5588,12 +5696,14 @@
       <c r="K68" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L68" s="2"/>
+      <c r="L68" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M68" s="5" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="N68" s="5" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="O68" s="2"/>
       <c r="P68" s="2"/>
@@ -5609,22 +5719,22 @@
         <v>70</v>
       </c>
       <c r="D69" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="E69" s="2" t="s">
         <v>484</v>
       </c>
-      <c r="E69" s="2" t="s">
-        <v>487</v>
-      </c>
       <c r="F69" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="J69" s="4">
         <v>46258</v>
@@ -5632,12 +5742,14 @@
       <c r="K69" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L69" s="2"/>
+      <c r="L69" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M69" s="5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="N69" s="5" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="O69" s="2"/>
       <c r="P69" s="2"/>
@@ -5647,28 +5759,28 @@
         <v>16</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="C70" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>22</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="J70" s="4">
         <v>46258</v>
@@ -5677,13 +5789,13 @@
         <v>49</v>
       </c>
       <c r="L70" s="2" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="M70" s="5" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="N70" s="5" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="O70" s="2"/>
       <c r="P70" s="2"/>
@@ -5693,22 +5805,22 @@
         <v>16</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>22</v>
@@ -5721,13 +5833,13 @@
         <v>49</v>
       </c>
       <c r="L71" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="M71" s="5" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="N71" s="5" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="O71" s="2"/>
       <c r="P71" s="2"/>
@@ -5737,28 +5849,28 @@
         <v>16</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="C72" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>41</v>
       </c>
       <c r="I72" s="3" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="J72" s="4">
         <v>46258</v>
@@ -5767,13 +5879,13 @@
         <v>49</v>
       </c>
       <c r="L72" s="2" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="M72" s="5" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="N72" s="5" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="O72" s="2"/>
       <c r="P72" s="2"/>
@@ -5783,28 +5895,28 @@
         <v>16</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="C73" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>56</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>41</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="J73" s="4">
         <v>46258</v>
@@ -5812,12 +5924,14 @@
       <c r="K73" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L73" s="2"/>
+      <c r="L73" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M73" s="5" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="N73" s="5" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="O73" s="2"/>
       <c r="P73" s="2"/>
@@ -5827,28 +5941,28 @@
         <v>16</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="C74" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="J74" s="4">
         <v>46258</v>
@@ -5856,12 +5970,14 @@
       <c r="K74" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L74" s="2"/>
+      <c r="L74" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M74" s="5" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="N74" s="5" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="O74" s="2"/>
       <c r="P74" s="2"/>
@@ -5871,28 +5987,28 @@
         <v>16</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="C75" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="J75" s="4">
         <v>46258</v>
@@ -5900,12 +6016,14 @@
       <c r="K75" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L75" s="2"/>
+      <c r="L75" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M75" s="5" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="N75" s="5" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="O75" s="2"/>
       <c r="P75" s="2"/>
@@ -5915,28 +6033,28 @@
         <v>16</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="J76" s="4">
         <v>46258</v>
@@ -5945,13 +6063,13 @@
         <v>49</v>
       </c>
       <c r="L76" s="2" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="M76" s="5" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="N76" s="5" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="O76" s="2"/>
       <c r="P76" s="2"/>
@@ -5967,19 +6085,19 @@
         <v>76</v>
       </c>
       <c r="D77" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="E77" s="2" t="s">
         <v>538</v>
       </c>
-      <c r="E77" s="2" t="s">
-        <v>541</v>
-      </c>
       <c r="F77" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="I77" s="3"/>
       <c r="J77" s="4">
@@ -5988,12 +6106,14 @@
       <c r="K77" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L77" s="2"/>
+      <c r="L77" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M77" s="5" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="N77" s="5" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="O77" s="2"/>
       <c r="P77" s="2"/>
@@ -6003,28 +6123,28 @@
         <v>16</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D78" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="F78" s="2" t="s">
         <v>544</v>
       </c>
-      <c r="E78" s="2" t="s">
-        <v>546</v>
-      </c>
-      <c r="F78" s="2" t="s">
-        <v>547</v>
-      </c>
       <c r="G78" s="2" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="J78" s="4">
         <v>46258</v>
@@ -6032,12 +6152,14 @@
       <c r="K78" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L78" s="2"/>
+      <c r="L78" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M78" s="5" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="N78" s="5" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="O78" s="2"/>
       <c r="P78" s="2"/>
@@ -6047,19 +6169,19 @@
         <v>16</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="G79" s="2" t="s">
         <v>25</v>
@@ -6068,7 +6190,7 @@
         <v>24</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="J79" s="4">
         <v>46258</v>
@@ -6076,12 +6198,14 @@
       <c r="K79" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L79" s="2"/>
+      <c r="L79" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M79" s="5" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="N79" s="5" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="O79" s="2"/>
       <c r="P79" s="2"/>
@@ -6091,16 +6215,16 @@
         <v>16</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>52</v>
@@ -6109,10 +6233,10 @@
         <v>53</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="I80" s="3" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="J80" s="4">
         <v>46258</v>
@@ -6121,13 +6245,13 @@
         <v>49</v>
       </c>
       <c r="L80" s="2" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="M80" s="5" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="N80" s="5" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="O80" s="2"/>
       <c r="P80" s="2"/>
@@ -6137,25 +6261,25 @@
         <v>16</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="G81" s="2" t="s">
         <v>29</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="I81" s="3"/>
       <c r="J81" s="4">
@@ -6164,12 +6288,14 @@
       <c r="K81" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L81" s="2"/>
+      <c r="L81" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M81" s="5" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="N81" s="5" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="O81" s="2"/>
       <c r="P81" s="2"/>
@@ -6179,25 +6305,25 @@
         <v>16</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="G82" s="2" t="s">
         <v>29</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="I82" s="3"/>
       <c r="J82" s="4">
@@ -6206,12 +6332,14 @@
       <c r="K82" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L82" s="2"/>
+      <c r="L82" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M82" s="5" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="N82" s="5" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="O82" s="2"/>
       <c r="P82" s="2"/>
@@ -6221,28 +6349,28 @@
         <v>16</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="H83" s="2" t="s">
         <v>24</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="J83" s="4">
         <v>46258</v>
@@ -6250,12 +6378,14 @@
       <c r="K83" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L83" s="2"/>
+      <c r="L83" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M83" s="5" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="N83" s="5" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="O83" s="2"/>
       <c r="P83" s="2"/>
@@ -6265,19 +6395,19 @@
         <v>16</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="G84" s="2" t="s">
         <v>38</v>
@@ -6286,7 +6416,7 @@
         <v>24</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="J84" s="4">
         <v>46258</v>
@@ -6294,12 +6424,14 @@
       <c r="K84" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L84" s="2"/>
+      <c r="L84" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M84" s="5" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="N84" s="5" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="O84" s="2"/>
       <c r="P84" s="2"/>
@@ -6315,13 +6447,13 @@
         <v>70</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>38</v>
@@ -6330,7 +6462,7 @@
         <v>24</v>
       </c>
       <c r="I85" s="3" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="J85" s="4">
         <v>46258</v>
@@ -6338,12 +6470,14 @@
       <c r="K85" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L85" s="2"/>
+      <c r="L85" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M85" s="5" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="N85" s="5" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="O85" s="2"/>
       <c r="P85" s="2"/>
@@ -6359,13 +6493,13 @@
         <v>70</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="G86" s="2" t="s">
         <v>38</v>
@@ -6374,7 +6508,7 @@
         <v>24</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="J86" s="4">
         <v>46258</v>
@@ -6382,12 +6516,14 @@
       <c r="K86" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L86" s="2"/>
+      <c r="L86" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M86" s="5" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="N86" s="5" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="O86" s="2"/>
       <c r="P86" s="2"/>
@@ -6397,19 +6533,19 @@
         <v>16</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="C87" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D87" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="E87" s="2" t="s">
         <v>585</v>
       </c>
-      <c r="E87" s="2" t="s">
-        <v>588</v>
-      </c>
       <c r="F87" s="2" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>37</v>
@@ -6418,7 +6554,7 @@
         <v>32</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="J87" s="4">
         <v>46258</v>
@@ -6427,13 +6563,13 @@
         <v>49</v>
       </c>
       <c r="L87" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="M87" s="5" t="s">
         <v>587</v>
       </c>
-      <c r="M87" s="5" t="s">
-        <v>590</v>
-      </c>
       <c r="N87" s="5" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="O87" s="2"/>
       <c r="P87" s="2"/>
@@ -6443,19 +6579,19 @@
         <v>16</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>37</v>
@@ -6464,7 +6600,7 @@
         <v>32</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="J88" s="4">
         <v>46258</v>
@@ -6472,12 +6608,14 @@
       <c r="K88" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L88" s="2"/>
+      <c r="L88" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M88" s="5" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="N88" s="5" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="O88" s="2"/>
       <c r="P88" s="2"/>
@@ -6487,28 +6625,28 @@
         <v>16</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="H89" s="2" t="s">
         <v>32</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="J89" s="4">
         <v>46258</v>
@@ -6516,12 +6654,14 @@
       <c r="K89" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L89" s="2"/>
+      <c r="L89" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M89" s="5" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="N89" s="5" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="O89" s="2"/>
       <c r="P89" s="2"/>
@@ -6531,28 +6671,28 @@
         <v>16</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="C90" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>57</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="J90" s="4">
         <v>46258</v>
@@ -6561,13 +6701,13 @@
         <v>49</v>
       </c>
       <c r="L90" s="2" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="M90" s="5" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="N90" s="5" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="O90" s="2"/>
       <c r="P90" s="2"/>
@@ -6577,28 +6717,28 @@
         <v>16</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="C91" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>57</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="J91" s="4">
         <v>46258</v>
@@ -6606,12 +6746,14 @@
       <c r="K91" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L91" s="2"/>
+      <c r="L91" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M91" s="5" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="N91" s="5" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="O91" s="2"/>
       <c r="P91" s="2"/>
@@ -6621,28 +6763,28 @@
         <v>16</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="C92" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D92" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="E92" s="2" t="s">
         <v>620</v>
       </c>
-      <c r="E92" s="2" t="s">
-        <v>623</v>
-      </c>
       <c r="F92" s="2" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="G92" s="2" t="s">
         <v>57</v>
       </c>
       <c r="H92" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="J92" s="4">
         <v>46258</v>
@@ -6651,13 +6793,13 @@
         <v>49</v>
       </c>
       <c r="L92" s="2" t="s">
+        <v>619</v>
+      </c>
+      <c r="M92" s="5" t="s">
+        <v>621</v>
+      </c>
+      <c r="N92" s="5" t="s">
         <v>622</v>
-      </c>
-      <c r="M92" s="5" t="s">
-        <v>624</v>
-      </c>
-      <c r="N92" s="5" t="s">
-        <v>625</v>
       </c>
       <c r="O92" s="2"/>
       <c r="P92" s="2"/>
@@ -6667,28 +6809,28 @@
         <v>16</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="C93" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>57</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="I93" s="3" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="J93" s="4">
         <v>46258</v>
@@ -6696,12 +6838,14 @@
       <c r="K93" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="L93" s="2"/>
+      <c r="L93" s="2" t="s">
+        <v>660</v>
+      </c>
       <c r="M93" s="5" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="N93" s="5" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="O93" s="2"/>
       <c r="P93" s="2"/>
@@ -6711,28 +6855,28 @@
         <v>16</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D94" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="G94" s="2" t="s">
         <v>633</v>
       </c>
-      <c r="E94" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="F94" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="G94" s="2" t="s">
-        <v>636</v>
-      </c>
       <c r="H94" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="I94" s="3" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="J94" s="4">
         <v>46258</v>
@@ -6741,13 +6885,13 @@
         <v>49</v>
       </c>
       <c r="L94" s="2" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="M94" s="5" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="N94" s="5" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="O94" s="2"/>
       <c r="P94" s="2"/>
@@ -6757,28 +6901,28 @@
         <v>16</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="C95" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="I95" s="3" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="J95" s="4">
         <v>46258</v>
@@ -6787,13 +6931,13 @@
         <v>60</v>
       </c>
       <c r="L95" s="2" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="M95" s="5" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="N95" s="5" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="O95" s="2"/>
       <c r="P95" s="2"/>
@@ -6803,19 +6947,19 @@
         <v>16</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="G96" s="2" t="s">
         <v>26</v>
@@ -6831,20 +6975,20 @@
         <v>61</v>
       </c>
       <c r="L96" s="2" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="M96" s="5" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="N96" s="5" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="O96" s="2"/>
       <c r="P96" s="2"/>
     </row>
     <row r="97" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="B97" s="2"/>
       <c r="C97" s="2" t="s">
@@ -6870,7 +7014,7 @@
     </row>
     <row r="98" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="B98" s="2"/>
       <c r="C98" s="2" t="s">
@@ -6896,7 +7040,7 @@
     </row>
     <row r="99" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="B99" s="2"/>
       <c r="C99" s="2" t="s">

</xml_diff>

<commit_message>
Publish September 4 CNG sources
</commit_message>
<xml_diff>
--- a/data/postes_d3s.xlsx
+++ b/data/postes_d3s.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olivierllinares/Documents/01_D3S 2025 2026/DNA 2025 2026/ED3S_Carte_V3_transfert_collegue-2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B640B58A-9182-D946-97A2-E71D7D1ABEB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BF37D9C-A720-1143-840C-2A954ADE0409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -160,7 +160,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1298" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="753">
   <si>
     <t>Actif ?</t>
   </si>
@@ -2414,6 +2414,12 @@
   </si>
   <si>
     <t>Fléché C Dautreppe</t>
+  </si>
+  <si>
+    <t>https://www.cng.sante.fr/sites/default/files/media/2026-09/joe_20260904_0206_0060.pdf</t>
+  </si>
+  <si>
+    <t>https://www.cng.sante.fr/sites/default/files/media/2026-09/joe_20260904_0206_0061.pdf</t>
   </si>
 </sst>
 </file>
@@ -2910,7 +2916,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>16</v>
       </c>
@@ -2939,9 +2945,11 @@
         <v>64</v>
       </c>
       <c r="J2" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K2" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L2" s="2" t="s">
         <v>633</v>
       </c>
@@ -2983,9 +2991,11 @@
         <v>71</v>
       </c>
       <c r="J3" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K3" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L3" s="2" t="s">
         <v>633</v>
       </c>
@@ -3027,9 +3037,11 @@
         <v>71</v>
       </c>
       <c r="J4" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K4" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L4" s="2" t="s">
         <v>633</v>
       </c>
@@ -3071,9 +3083,11 @@
         <v>76</v>
       </c>
       <c r="J5" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K5" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L5" s="2" t="s">
         <v>633</v>
       </c>
@@ -3115,9 +3129,11 @@
         <v>83</v>
       </c>
       <c r="J6" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K6" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L6" s="2" t="s">
         <v>749</v>
       </c>
@@ -3159,9 +3175,11 @@
         <v>93</v>
       </c>
       <c r="J7" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K7" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L7" s="2" t="s">
         <v>112</v>
       </c>
@@ -3201,9 +3219,11 @@
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K8" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L8" s="2" t="s">
         <v>633</v>
       </c>
@@ -3216,7 +3236,7 @@
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
     </row>
-    <row r="9" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -3245,9 +3265,11 @@
         <v>103</v>
       </c>
       <c r="J9" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K9" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L9" s="2" t="s">
         <v>633</v>
       </c>
@@ -3289,9 +3311,11 @@
         <v>638</v>
       </c>
       <c r="J10" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K10" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L10" s="2" t="s">
         <v>633</v>
       </c>
@@ -3304,7 +3328,7 @@
       <c r="O10" s="2"/>
       <c r="P10" s="2"/>
     </row>
-    <row r="11" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>16</v>
       </c>
@@ -3333,9 +3357,11 @@
         <v>106</v>
       </c>
       <c r="J11" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K11" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L11" s="2" t="s">
         <v>116</v>
       </c>
@@ -3377,9 +3403,11 @@
         <v>109</v>
       </c>
       <c r="J12" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K12" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L12" s="2" t="s">
         <v>633</v>
       </c>
@@ -3392,7 +3420,7 @@
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
     </row>
-    <row r="13" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
@@ -3421,9 +3449,11 @@
         <v>117</v>
       </c>
       <c r="J13" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K13" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L13" s="2" t="s">
         <v>633</v>
       </c>
@@ -3465,9 +3495,11 @@
         <v>122</v>
       </c>
       <c r="J14" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K14" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L14" s="2" t="s">
         <v>633</v>
       </c>
@@ -3509,9 +3541,11 @@
         <v>129</v>
       </c>
       <c r="J15" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K15" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L15" s="2" t="s">
         <v>633</v>
       </c>
@@ -3553,9 +3587,11 @@
         <v>644</v>
       </c>
       <c r="J16" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K16" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L16" s="2" t="s">
         <v>633</v>
       </c>
@@ -3568,7 +3604,7 @@
       <c r="O16" s="2"/>
       <c r="P16" s="2"/>
     </row>
-    <row r="17" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -3597,9 +3633,11 @@
         <v>132</v>
       </c>
       <c r="J17" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K17" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L17" s="2" t="s">
         <v>136</v>
       </c>
@@ -3641,9 +3679,11 @@
         <v>658</v>
       </c>
       <c r="J18" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K18" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L18" s="2" t="s">
         <v>633</v>
       </c>
@@ -3683,9 +3723,11 @@
       </c>
       <c r="I19" s="3"/>
       <c r="J19" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K19" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L19" s="2" t="s">
         <v>633</v>
       </c>
@@ -3727,9 +3769,11 @@
         <v>141</v>
       </c>
       <c r="J20" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K20" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L20" s="2" t="s">
         <v>633</v>
       </c>
@@ -3742,7 +3786,7 @@
       <c r="O20" s="2"/>
       <c r="P20" s="2"/>
     </row>
-    <row r="21" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>16</v>
       </c>
@@ -3771,9 +3815,11 @@
         <v>35</v>
       </c>
       <c r="J21" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K21" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L21" s="2" t="s">
         <v>633</v>
       </c>
@@ -3815,9 +3861,11 @@
         <v>141</v>
       </c>
       <c r="J22" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K22" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L22" s="2" t="s">
         <v>633</v>
       </c>
@@ -3859,9 +3907,11 @@
         <v>156</v>
       </c>
       <c r="J23" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K23" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L23" s="2" t="s">
         <v>633</v>
       </c>
@@ -3874,7 +3924,7 @@
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
     </row>
-    <row r="24" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>16</v>
       </c>
@@ -3903,9 +3953,11 @@
         <v>162</v>
       </c>
       <c r="J24" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K24" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L24" s="2" t="s">
         <v>633</v>
       </c>
@@ -3918,7 +3970,7 @@
       <c r="O24" s="2"/>
       <c r="P24" s="2"/>
     </row>
-    <row r="25" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>16</v>
       </c>
@@ -3947,9 +3999,11 @@
         <v>167</v>
       </c>
       <c r="J25" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K25" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L25" s="2" t="s">
         <v>633</v>
       </c>
@@ -3991,9 +4045,11 @@
         <v>664</v>
       </c>
       <c r="J26" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K26" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L26" s="2" t="s">
         <v>633</v>
       </c>
@@ -4035,9 +4091,11 @@
         <v>172</v>
       </c>
       <c r="J27" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K27" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L27" s="2" t="s">
         <v>633</v>
       </c>
@@ -4050,7 +4108,7 @@
       <c r="O27" s="2"/>
       <c r="P27" s="2"/>
     </row>
-    <row r="28" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>16</v>
       </c>
@@ -4079,9 +4137,11 @@
         <v>179</v>
       </c>
       <c r="J28" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K28" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L28" s="2" t="s">
         <v>633</v>
       </c>
@@ -4094,7 +4154,7 @@
       <c r="O28" s="2"/>
       <c r="P28" s="2"/>
     </row>
-    <row r="29" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>16</v>
       </c>
@@ -4123,9 +4183,11 @@
         <v>182</v>
       </c>
       <c r="J29" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K29" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L29" s="2" t="s">
         <v>633</v>
       </c>
@@ -4138,7 +4200,7 @@
       <c r="O29" s="2"/>
       <c r="P29" s="2"/>
     </row>
-    <row r="30" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>16</v>
       </c>
@@ -4167,9 +4229,11 @@
         <v>190</v>
       </c>
       <c r="J30" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K30" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L30" s="2" t="s">
         <v>633</v>
       </c>
@@ -4182,7 +4246,7 @@
       <c r="O30" s="2"/>
       <c r="P30" s="2"/>
     </row>
-    <row r="31" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>16</v>
       </c>
@@ -4211,9 +4275,11 @@
         <v>270000367</v>
       </c>
       <c r="J31" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K31" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L31" s="2" t="s">
         <v>633</v>
       </c>
@@ -4226,7 +4292,7 @@
       <c r="O31" s="2"/>
       <c r="P31" s="2"/>
     </row>
-    <row r="32" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>16</v>
       </c>
@@ -4255,9 +4321,11 @@
         <v>203</v>
       </c>
       <c r="J32" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K32" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L32" s="2" t="s">
         <v>633</v>
       </c>
@@ -4270,7 +4338,7 @@
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
     </row>
-    <row r="33" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>16</v>
       </c>
@@ -4299,9 +4367,11 @@
         <v>669</v>
       </c>
       <c r="J33" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K33" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L33" s="2" t="s">
         <v>633</v>
       </c>
@@ -4343,9 +4413,11 @@
         <v>673</v>
       </c>
       <c r="J34" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K34" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L34" s="2" t="s">
         <v>633</v>
       </c>
@@ -4358,7 +4430,7 @@
       <c r="O34" s="2"/>
       <c r="P34" s="2"/>
     </row>
-    <row r="35" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>16</v>
       </c>
@@ -4387,9 +4459,11 @@
         <v>213</v>
       </c>
       <c r="J35" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K35" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L35" s="2" t="s">
         <v>633</v>
       </c>
@@ -4402,7 +4476,7 @@
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
     </row>
-    <row r="36" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>16</v>
       </c>
@@ -4431,9 +4505,11 @@
         <v>221</v>
       </c>
       <c r="J36" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K36" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L36" s="2" t="s">
         <v>633</v>
       </c>
@@ -4473,9 +4549,11 @@
       </c>
       <c r="I37" s="3"/>
       <c r="J37" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K37" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L37" s="2" t="s">
         <v>229</v>
       </c>
@@ -4517,9 +4595,11 @@
         <v>230</v>
       </c>
       <c r="J38" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K38" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L38" s="2" t="s">
         <v>633</v>
       </c>
@@ -4561,9 +4641,11 @@
         <v>231</v>
       </c>
       <c r="J39" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K39" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L39" s="2" t="s">
         <v>633</v>
       </c>
@@ -4605,9 +4687,11 @@
         <v>243</v>
       </c>
       <c r="J40" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K40" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L40" s="2" t="s">
         <v>633</v>
       </c>
@@ -4649,9 +4733,11 @@
         <v>245</v>
       </c>
       <c r="J41" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K41" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L41" s="2" t="s">
         <v>633</v>
       </c>
@@ -4693,9 +4779,11 @@
         <v>683</v>
       </c>
       <c r="J42" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K42" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L42" s="2" t="s">
         <v>633</v>
       </c>
@@ -4737,9 +4825,11 @@
         <v>679</v>
       </c>
       <c r="J43" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K43" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L43" s="2" t="s">
         <v>633</v>
       </c>
@@ -4781,9 +4871,11 @@
         <v>246</v>
       </c>
       <c r="J44" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K44" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L44" s="2" t="s">
         <v>633</v>
       </c>
@@ -4796,7 +4888,7 @@
       <c r="O44" s="2"/>
       <c r="P44" s="2"/>
     </row>
-    <row r="45" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>16</v>
       </c>
@@ -4823,9 +4915,11 @@
       </c>
       <c r="I45" s="3"/>
       <c r="J45" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K45" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L45" s="2" t="s">
         <v>633</v>
       </c>
@@ -4867,9 +4961,11 @@
         <v>689</v>
       </c>
       <c r="J46" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K46" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L46" s="2" t="s">
         <v>633</v>
       </c>
@@ -4882,7 +4978,7 @@
       <c r="O46" s="2"/>
       <c r="P46" s="2"/>
     </row>
-    <row r="47" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>16</v>
       </c>
@@ -4911,9 +5007,11 @@
         <v>269</v>
       </c>
       <c r="J47" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K47" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L47" s="2" t="s">
         <v>633</v>
       </c>
@@ -4955,9 +5053,11 @@
         <v>276</v>
       </c>
       <c r="J48" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K48" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L48" s="2" t="s">
         <v>282</v>
       </c>
@@ -4999,9 +5099,11 @@
         <v>276</v>
       </c>
       <c r="J49" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K49" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L49" s="2" t="s">
         <v>633</v>
       </c>
@@ -5043,9 +5145,11 @@
         <v>292</v>
       </c>
       <c r="J50" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K50" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L50" s="2" t="s">
         <v>633</v>
       </c>
@@ -5058,7 +5162,7 @@
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
     </row>
-    <row r="51" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>16</v>
       </c>
@@ -5087,9 +5191,11 @@
         <v>298</v>
       </c>
       <c r="J51" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K51" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L51" s="2" t="s">
         <v>633</v>
       </c>
@@ -5129,9 +5235,11 @@
         <v>703</v>
       </c>
       <c r="J52" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K52" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L52" s="2" t="s">
         <v>633</v>
       </c>
@@ -5171,9 +5279,11 @@
         <v>702</v>
       </c>
       <c r="J53" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K53" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L53" s="2" t="s">
         <v>633</v>
       </c>
@@ -5215,9 +5325,11 @@
         <v>305</v>
       </c>
       <c r="J54" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K54" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L54" s="2" t="s">
         <v>633</v>
       </c>
@@ -5230,7 +5342,7 @@
       <c r="O54" s="2"/>
       <c r="P54" s="2"/>
     </row>
-    <row r="55" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>16</v>
       </c>
@@ -5259,9 +5371,11 @@
         <v>312</v>
       </c>
       <c r="J55" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K55" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L55" s="2" t="s">
         <v>633</v>
       </c>
@@ -5301,9 +5415,11 @@
         <v>708</v>
       </c>
       <c r="J56" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K56" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L56" s="2" t="s">
         <v>633</v>
       </c>
@@ -5316,7 +5432,7 @@
       <c r="O56" s="2"/>
       <c r="P56" s="2"/>
     </row>
-    <row r="57" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>16</v>
       </c>
@@ -5345,9 +5461,11 @@
         <v>317</v>
       </c>
       <c r="J57" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K57" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L57" s="2" t="s">
         <v>323</v>
       </c>
@@ -5360,7 +5478,7 @@
       <c r="O57" s="2"/>
       <c r="P57" s="2"/>
     </row>
-    <row r="58" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>16</v>
       </c>
@@ -5389,9 +5507,11 @@
         <v>325</v>
       </c>
       <c r="J58" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K58" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L58" s="2" t="s">
         <v>633</v>
       </c>
@@ -5404,7 +5524,7 @@
       <c r="O58" s="2"/>
       <c r="P58" s="2"/>
     </row>
-    <row r="59" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>16</v>
       </c>
@@ -5433,9 +5553,11 @@
         <v>332</v>
       </c>
       <c r="J59" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K59" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L59" s="2" t="s">
         <v>633</v>
       </c>
@@ -5477,9 +5599,11 @@
         <v>337</v>
       </c>
       <c r="J60" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K60" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L60" s="2" t="s">
         <v>633</v>
       </c>
@@ -5492,7 +5616,7 @@
       <c r="O60" s="2"/>
       <c r="P60" s="2"/>
     </row>
-    <row r="61" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>16</v>
       </c>
@@ -5521,9 +5645,11 @@
         <v>344</v>
       </c>
       <c r="J61" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K61" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L61" s="2" t="s">
         <v>633</v>
       </c>
@@ -5536,7 +5662,7 @@
       <c r="O61" s="2"/>
       <c r="P61" s="2"/>
     </row>
-    <row r="62" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>16</v>
       </c>
@@ -5565,9 +5691,11 @@
         <v>350</v>
       </c>
       <c r="J62" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K62" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L62" s="2" t="s">
         <v>633</v>
       </c>
@@ -5609,9 +5737,11 @@
         <v>362</v>
       </c>
       <c r="J63" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K63" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L63" s="2" t="s">
         <v>633</v>
       </c>
@@ -5653,9 +5783,11 @@
         <v>364</v>
       </c>
       <c r="J64" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K64" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L64" s="2" t="s">
         <v>372</v>
       </c>
@@ -5668,7 +5800,7 @@
       <c r="O64" s="2"/>
       <c r="P64" s="2"/>
     </row>
-    <row r="65" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>16</v>
       </c>
@@ -5695,9 +5827,11 @@
       </c>
       <c r="I65" s="3"/>
       <c r="J65" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K65" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L65" s="2" t="s">
         <v>633</v>
       </c>
@@ -5710,7 +5844,7 @@
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
     </row>
-    <row r="66" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>16</v>
       </c>
@@ -5739,9 +5873,11 @@
         <v>373</v>
       </c>
       <c r="J66" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K66" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L66" s="2" t="s">
         <v>633</v>
       </c>
@@ -5783,9 +5919,11 @@
         <v>379</v>
       </c>
       <c r="J67" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K67" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K67" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L67" s="2" t="s">
         <v>384</v>
       </c>
@@ -5827,9 +5965,11 @@
         <v>387</v>
       </c>
       <c r="J68" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K68" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K68" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L68" s="2" t="s">
         <v>392</v>
       </c>
@@ -5871,9 +6011,11 @@
         <v>395</v>
       </c>
       <c r="J69" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K69" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L69" s="2" t="s">
         <v>633</v>
       </c>
@@ -5886,7 +6028,7 @@
       <c r="O69" s="2"/>
       <c r="P69" s="2"/>
     </row>
-    <row r="70" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>16</v>
       </c>
@@ -5915,9 +6057,11 @@
         <v>401</v>
       </c>
       <c r="J70" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K70" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K70" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L70" s="2" t="s">
         <v>633</v>
       </c>
@@ -5930,7 +6074,7 @@
       <c r="O70" s="2"/>
       <c r="P70" s="2"/>
     </row>
-    <row r="71" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>16</v>
       </c>
@@ -5959,9 +6103,11 @@
         <v>406</v>
       </c>
       <c r="J71" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K71" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K71" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L71" s="2" t="s">
         <v>633</v>
       </c>
@@ -5974,7 +6120,7 @@
       <c r="O71" s="2"/>
       <c r="P71" s="2"/>
     </row>
-    <row r="72" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>16</v>
       </c>
@@ -6003,9 +6149,11 @@
         <v>413</v>
       </c>
       <c r="J72" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K72" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K72" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L72" s="2" t="s">
         <v>417</v>
       </c>
@@ -6018,7 +6166,7 @@
       <c r="O72" s="2"/>
       <c r="P72" s="2"/>
     </row>
-    <row r="73" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>16</v>
       </c>
@@ -6047,9 +6195,11 @@
         <v>420</v>
       </c>
       <c r="J73" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K73" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K73" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L73" s="2" t="s">
         <v>633</v>
       </c>
@@ -6091,9 +6241,11 @@
         <v>427</v>
       </c>
       <c r="J74" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K74" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K74" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L74" s="2" t="s">
         <v>433</v>
       </c>
@@ -6135,9 +6287,11 @@
         <v>427</v>
       </c>
       <c r="J75" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K75" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K75" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L75" s="2" t="s">
         <v>633</v>
       </c>
@@ -6179,9 +6333,11 @@
         <v>434</v>
       </c>
       <c r="J76" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K76" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K76" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L76" s="2" t="s">
         <v>633</v>
       </c>
@@ -6194,7 +6350,7 @@
       <c r="O76" s="2"/>
       <c r="P76" s="2"/>
     </row>
-    <row r="77" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>16</v>
       </c>
@@ -6223,9 +6379,11 @@
         <v>442</v>
       </c>
       <c r="J77" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K77" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K77" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L77" s="2" t="s">
         <v>633</v>
       </c>
@@ -6238,7 +6396,7 @@
       <c r="O77" s="2"/>
       <c r="P77" s="2"/>
     </row>
-    <row r="78" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>16</v>
       </c>
@@ -6267,9 +6425,11 @@
         <v>448</v>
       </c>
       <c r="J78" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K78" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K78" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L78" s="2" t="s">
         <v>633</v>
       </c>
@@ -6311,9 +6471,11 @@
         <v>455</v>
       </c>
       <c r="J79" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K79" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K79" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L79" s="2" t="s">
         <v>633</v>
       </c>
@@ -6326,7 +6488,7 @@
       <c r="O79" s="2"/>
       <c r="P79" s="2"/>
     </row>
-    <row r="80" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>16</v>
       </c>
@@ -6355,9 +6517,11 @@
         <v>460</v>
       </c>
       <c r="J80" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K80" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K80" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L80" s="2" t="s">
         <v>465</v>
       </c>
@@ -6397,9 +6561,11 @@
       </c>
       <c r="I81" s="3"/>
       <c r="J81" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K81" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K81" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L81" s="2" t="s">
         <v>471</v>
       </c>
@@ -6412,7 +6578,7 @@
       <c r="O81" s="2"/>
       <c r="P81" s="2"/>
     </row>
-    <row r="82" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>16</v>
       </c>
@@ -6441,9 +6607,11 @@
         <v>475</v>
       </c>
       <c r="J82" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K82" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K82" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L82" s="2" t="s">
         <v>479</v>
       </c>
@@ -6485,9 +6653,11 @@
         <v>475</v>
       </c>
       <c r="J83" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K83" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K83" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L83" s="2" t="s">
         <v>633</v>
       </c>
@@ -6529,9 +6699,11 @@
         <v>488</v>
       </c>
       <c r="J84" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K84" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K84" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L84" s="2" t="s">
         <v>633</v>
       </c>
@@ -6573,9 +6745,11 @@
         <v>496</v>
       </c>
       <c r="J85" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K85" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K85" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L85" s="2" t="s">
         <v>750</v>
       </c>
@@ -6617,9 +6791,11 @@
         <v>503</v>
       </c>
       <c r="J86" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K86" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K86" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L86" s="2" t="s">
         <v>508</v>
       </c>
@@ -6632,7 +6808,7 @@
       <c r="O86" s="2"/>
       <c r="P86" s="2"/>
     </row>
-    <row r="87" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>16</v>
       </c>
@@ -6659,9 +6835,11 @@
       </c>
       <c r="I87" s="3"/>
       <c r="J87" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K87" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K87" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L87" s="2" t="s">
         <v>633</v>
       </c>
@@ -6703,9 +6881,11 @@
         <v>514</v>
       </c>
       <c r="J88" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K88" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K88" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L88" s="2" t="s">
         <v>633</v>
       </c>
@@ -6747,9 +6927,11 @@
         <v>522</v>
       </c>
       <c r="J89" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K89" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K89" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L89" s="2" t="s">
         <v>633</v>
       </c>
@@ -6762,7 +6944,7 @@
       <c r="O89" s="2"/>
       <c r="P89" s="2"/>
     </row>
-    <row r="90" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>16</v>
       </c>
@@ -6791,9 +6973,11 @@
         <v>528</v>
       </c>
       <c r="J90" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K90" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K90" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L90" s="2" t="s">
         <v>529</v>
       </c>
@@ -6806,7 +6990,7 @@
       <c r="O90" s="2"/>
       <c r="P90" s="2"/>
     </row>
-    <row r="91" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>16</v>
       </c>
@@ -6833,9 +7017,11 @@
       </c>
       <c r="I91" s="3"/>
       <c r="J91" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K91" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K91" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L91" s="2" t="s">
         <v>633</v>
       </c>
@@ -6848,7 +7034,7 @@
       <c r="O91" s="2"/>
       <c r="P91" s="2"/>
     </row>
-    <row r="92" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
         <v>16</v>
       </c>
@@ -6875,9 +7061,11 @@
       </c>
       <c r="I92" s="3"/>
       <c r="J92" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K92" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K92" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L92" s="2" t="s">
         <v>633</v>
       </c>
@@ -6890,7 +7078,7 @@
       <c r="O92" s="2"/>
       <c r="P92" s="2"/>
     </row>
-    <row r="93" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
         <v>16</v>
       </c>
@@ -6919,9 +7107,11 @@
         <v>537</v>
       </c>
       <c r="J93" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K93" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K93" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L93" s="2" t="s">
         <v>633</v>
       </c>
@@ -6963,9 +7153,11 @@
         <v>544</v>
       </c>
       <c r="J94" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K94" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K94" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L94" s="2" t="s">
         <v>633</v>
       </c>
@@ -6978,7 +7170,7 @@
       <c r="O94" s="2"/>
       <c r="P94" s="2"/>
     </row>
-    <row r="95" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>16</v>
       </c>
@@ -7007,9 +7199,11 @@
         <v>550</v>
       </c>
       <c r="J95" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K95" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K95" s="2" t="s">
+        <v>752</v>
+      </c>
       <c r="L95" s="2" t="s">
         <v>633</v>
       </c>
@@ -7051,9 +7245,11 @@
         <v>717</v>
       </c>
       <c r="J96" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K96" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K96" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L96" s="2" t="s">
         <v>633</v>
       </c>
@@ -7095,9 +7291,11 @@
         <v>555</v>
       </c>
       <c r="J97" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K97" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K97" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L97" s="2" t="s">
         <v>558</v>
       </c>
@@ -7139,9 +7337,11 @@
         <v>563</v>
       </c>
       <c r="J98" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K98" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K98" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L98" s="2" t="s">
         <v>633</v>
       </c>
@@ -7183,9 +7383,11 @@
         <v>569</v>
       </c>
       <c r="J99" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K99" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K99" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L99" s="2" t="s">
         <v>633</v>
       </c>
@@ -7227,9 +7429,11 @@
         <v>577</v>
       </c>
       <c r="J100" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K100" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K100" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L100" s="2" t="s">
         <v>583</v>
       </c>
@@ -7242,7 +7446,7 @@
       <c r="O100" s="2"/>
       <c r="P100" s="2"/>
     </row>
-    <row r="101" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
         <v>16</v>
       </c>
@@ -7271,9 +7475,11 @@
         <v>584</v>
       </c>
       <c r="J101" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K101" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K101" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L101" s="2" t="s">
         <v>633</v>
       </c>
@@ -7315,9 +7521,11 @@
         <v>590</v>
       </c>
       <c r="J102" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K102" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K102" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L102" s="2" t="s">
         <v>593</v>
       </c>
@@ -7359,9 +7567,11 @@
         <v>597</v>
       </c>
       <c r="J103" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K103" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K103" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L103" s="2" t="s">
         <v>633</v>
       </c>
@@ -7403,9 +7613,11 @@
         <v>603</v>
       </c>
       <c r="J104" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K104" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K104" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L104" s="2" t="s">
         <v>610</v>
       </c>
@@ -7447,9 +7659,11 @@
         <v>611</v>
       </c>
       <c r="J105" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K105" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K105" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L105" s="2" t="s">
         <v>617</v>
       </c>
@@ -7491,9 +7705,11 @@
         <v>725</v>
       </c>
       <c r="J106" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K106" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K106" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L106" s="2" t="s">
         <v>633</v>
       </c>
@@ -7533,9 +7749,11 @@
       </c>
       <c r="I107" s="3"/>
       <c r="J107" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K107" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K107" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L107" s="2" t="s">
         <v>633</v>
       </c>
@@ -7577,9 +7795,11 @@
         <v>732</v>
       </c>
       <c r="J108" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K108" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K108" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L108" s="2" t="s">
         <v>630</v>
       </c>
@@ -7621,9 +7841,11 @@
         <v>731</v>
       </c>
       <c r="J109" s="4">
-        <v>46268</v>
-      </c>
-      <c r="K109" s="2"/>
+        <v>46269</v>
+      </c>
+      <c r="K109" s="2" t="s">
+        <v>751</v>
+      </c>
       <c r="L109" s="2" t="s">
         <v>735</v>
       </c>

</xml_diff>